<commit_message>
refactor: ProjectTable 삭제 — PivotProjectTable로 완전 교체
ProjectTable.tsx는 PivotProjectTable로 교체되었으며 더 이상 사용되지 않음.
TypeScript 검증 및 모든 단위 테스트 통과 확인.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/공사현황.xlsx
+++ b/공사현황.xlsx
@@ -1275,7 +1275,7 @@
 
 <file path=xl/worksheets/sheet0.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G298"/>
+  <dimension ref="A1:G300"/>
   <cols>
     <col min="1" max="1" width="11.43" customWidth="1"/>
     <col min="2" max="2" width="11.43" customWidth="1"/>
@@ -3242,49 +3242,49 @@
       </c>
     </row>
     <row r="86" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A86" s="3" t="s">
+      <c r="A86" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B86" s="7">
-        <v>46184</v>
-      </c>
-      <c r="C86" s="9" t="n">
-        <v>54.00</v>
-      </c>
-      <c r="D86" s="3" t="s">
+      <c r="B86" s="6">
+        <v>46187</v>
+      </c>
+      <c r="C86" s="8" t="n">
+        <v>100.00</v>
+      </c>
+      <c r="D86" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="E86" s="12" t="n">
-        <v>4035280.68</v>
-      </c>
-      <c r="F86" s="12" t="n">
-        <v>3743271.28</v>
-      </c>
-      <c r="G86" s="12" t="n">
-        <v>292009.40</v>
+      <c r="E86" s="11" t="n">
+        <v>7472742.00</v>
+      </c>
+      <c r="F86" s="11" t="n">
+        <v>7550142.56</v>
+      </c>
+      <c r="G86" s="11" t="n">
+        <v>-77400.56</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="16.5" customHeight="1">
       <c r="A87" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B87" s="6">
-        <v>46128</v>
+        <v>46184</v>
       </c>
       <c r="C87" s="8" t="n">
-        <v>90.00</v>
+        <v>54.00</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E87" s="11" t="n">
-        <v>12087832.50</v>
+        <v>7472742.00</v>
       </c>
       <c r="F87" s="11" t="n">
-        <v>13481578.20</v>
+        <v>7550142.56</v>
       </c>
       <c r="G87" s="11" t="n">
-        <v>-1393745.70</v>
+        <v>-77400.56</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="16.5" customHeight="1">
@@ -3292,10 +3292,10 @@
         <v>50</v>
       </c>
       <c r="B88" s="6">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="C88" s="8" t="n">
-        <v>50.00</v>
+        <v>90.00</v>
       </c>
       <c r="D88" s="2" t="s">
         <v>180</v>
@@ -3315,10 +3315,10 @@
         <v>50</v>
       </c>
       <c r="B89" s="6">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="C89" s="8" t="n">
-        <v>10.00</v>
+        <v>50.00</v>
       </c>
       <c r="D89" s="2" t="s">
         <v>180</v>
@@ -3335,140 +3335,140 @@
     </row>
     <row r="90" spans="1:7" ht="16.5" customHeight="1">
       <c r="A90" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B90" s="6">
+        <v>46126</v>
+      </c>
+      <c r="C90" s="8" t="n">
+        <v>10.00</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E90" s="11" t="n">
+        <v>12087832.50</v>
+      </c>
+      <c r="F90" s="11" t="n">
+        <v>13481578.20</v>
+      </c>
+      <c r="G90" s="11" t="n">
+        <v>-1393745.70</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A91" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B90" s="6">
+      <c r="B91" s="6">
         <v>46036</v>
       </c>
-      <c r="C90" s="8" t="n">
+      <c r="C91" s="8" t="n">
         <v>95.00</v>
       </c>
-      <c r="D90" s="2" t="s">
+      <c r="D91" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="E90" s="11" t="n">
+      <c r="E91" s="11" t="n">
         <v>181803.40</v>
       </c>
-      <c r="F90" s="11" t="n">
+      <c r="F91" s="11" t="n">
         <v>420208.91</v>
       </c>
-      <c r="G90" s="11" t="n">
+      <c r="G91" s="11" t="n">
         <v>-238405.51</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A91" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B91" s="7">
-        <v>46035</v>
-      </c>
-      <c r="C91" s="9" t="n">
-        <v>95.00</v>
-      </c>
-      <c r="D91" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="E91" s="12" t="n">
-        <v>788788.41</v>
-      </c>
-      <c r="F91" s="12" t="n">
-        <v>420208.91</v>
-      </c>
-      <c r="G91" s="12" t="n">
-        <v>368579.50</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="16.5" customHeight="1">
       <c r="A92" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B92" s="7">
-        <v>46107</v>
+        <v>46035</v>
       </c>
       <c r="C92" s="9" t="n">
         <v>95.00</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E92" s="12" t="n">
-        <v>599108.11</v>
+        <v>788788.41</v>
       </c>
       <c r="F92" s="12" t="n">
         <v>420208.91</v>
       </c>
       <c r="G92" s="12" t="n">
+        <v>368579.50</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A93" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B93" s="7">
+        <v>46107</v>
+      </c>
+      <c r="C93" s="9" t="n">
+        <v>95.00</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="E93" s="12" t="n">
+        <v>599108.11</v>
+      </c>
+      <c r="F93" s="12" t="n">
+        <v>420208.91</v>
+      </c>
+      <c r="G93" s="12" t="n">
         <v>178899.20</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A93" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B93" s="6">
-        <v>46056</v>
-      </c>
-      <c r="C93" s="8" t="n">
-        <v>95.00</v>
-      </c>
-      <c r="D93" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="E93" s="11" t="n">
-        <v>195625.92</v>
-      </c>
-      <c r="F93" s="11" t="n">
-        <v>1260626.73</v>
-      </c>
-      <c r="G93" s="11" t="n">
-        <v>-1065000.81</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="16.5" customHeight="1">
       <c r="A94" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B94" s="6">
-        <v>46107</v>
+        <v>46056</v>
       </c>
       <c r="C94" s="8" t="n">
         <v>95.00</v>
       </c>
       <c r="D94" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E94" s="11" t="n">
+        <v>195625.92</v>
+      </c>
+      <c r="F94" s="11" t="n">
+        <v>1260626.73</v>
+      </c>
+      <c r="G94" s="11" t="n">
+        <v>-1065000.81</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A95" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B95" s="6">
+        <v>46107</v>
+      </c>
+      <c r="C95" s="8" t="n">
+        <v>95.00</v>
+      </c>
+      <c r="D95" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="E94" s="11" t="n">
+      <c r="E95" s="11" t="n">
         <v>65578.87</v>
       </c>
-      <c r="F94" s="11" t="n">
+      <c r="F95" s="11" t="n">
         <v>168083.56</v>
       </c>
-      <c r="G94" s="11" t="n">
+      <c r="G95" s="11" t="n">
         <v>-102504.69</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A95" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B95" s="7">
-        <v>46065</v>
-      </c>
-      <c r="C95" s="9" t="n">
-        <v>96.00</v>
-      </c>
-      <c r="D95" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="E95" s="12" t="n">
-        <v>94079929.55</v>
-      </c>
-      <c r="F95" s="12" t="n">
-        <v>58829247.40</v>
-      </c>
-      <c r="G95" s="12" t="n">
-        <v>35250682.15</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="16.5" customHeight="1">
@@ -3476,10 +3476,10 @@
         <v>56</v>
       </c>
       <c r="B96" s="7">
-        <v>46064</v>
+        <v>46065</v>
       </c>
       <c r="C96" s="9" t="n">
-        <v>94.00</v>
+        <v>96.00</v>
       </c>
       <c r="D96" s="3" t="s">
         <v>186</v>
@@ -3499,10 +3499,10 @@
         <v>56</v>
       </c>
       <c r="B97" s="7">
-        <v>46063</v>
+        <v>46064</v>
       </c>
       <c r="C97" s="9" t="n">
-        <v>92.00</v>
+        <v>94.00</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>186</v>
@@ -3522,10 +3522,10 @@
         <v>56</v>
       </c>
       <c r="B98" s="7">
-        <v>46062</v>
+        <v>46063</v>
       </c>
       <c r="C98" s="9" t="n">
-        <v>90.00</v>
+        <v>92.00</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>186</v>
@@ -3545,10 +3545,10 @@
         <v>56</v>
       </c>
       <c r="B99" s="7">
-        <v>46059</v>
+        <v>46062</v>
       </c>
       <c r="C99" s="9" t="n">
-        <v>87.00</v>
+        <v>90.00</v>
       </c>
       <c r="D99" s="3" t="s">
         <v>186</v>
@@ -3568,10 +3568,10 @@
         <v>56</v>
       </c>
       <c r="B100" s="7">
-        <v>46058</v>
+        <v>46059</v>
       </c>
       <c r="C100" s="9" t="n">
-        <v>79.00</v>
+        <v>87.00</v>
       </c>
       <c r="D100" s="3" t="s">
         <v>186</v>
@@ -3591,10 +3591,10 @@
         <v>56</v>
       </c>
       <c r="B101" s="7">
-        <v>46057</v>
+        <v>46058</v>
       </c>
       <c r="C101" s="9" t="n">
-        <v>67.00</v>
+        <v>79.00</v>
       </c>
       <c r="D101" s="3" t="s">
         <v>186</v>
@@ -3614,10 +3614,10 @@
         <v>56</v>
       </c>
       <c r="B102" s="7">
-        <v>46056</v>
+        <v>46057</v>
       </c>
       <c r="C102" s="9" t="n">
-        <v>55.00</v>
+        <v>67.00</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>186</v>
@@ -3637,10 +3637,10 @@
         <v>56</v>
       </c>
       <c r="B103" s="7">
-        <v>46055</v>
+        <v>46056</v>
       </c>
       <c r="C103" s="9" t="n">
-        <v>50.00</v>
+        <v>55.00</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>186</v>
@@ -3660,10 +3660,10 @@
         <v>56</v>
       </c>
       <c r="B104" s="7">
-        <v>46052</v>
+        <v>46055</v>
       </c>
       <c r="C104" s="9" t="n">
-        <v>42.00</v>
+        <v>50.00</v>
       </c>
       <c r="D104" s="3" t="s">
         <v>186</v>
@@ -3683,10 +3683,10 @@
         <v>56</v>
       </c>
       <c r="B105" s="7">
-        <v>46051</v>
+        <v>46052</v>
       </c>
       <c r="C105" s="9" t="n">
-        <v>32.00</v>
+        <v>42.00</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>186</v>
@@ -3706,10 +3706,10 @@
         <v>56</v>
       </c>
       <c r="B106" s="7">
-        <v>46050</v>
+        <v>46051</v>
       </c>
       <c r="C106" s="9" t="n">
-        <v>25.00</v>
+        <v>32.00</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>186</v>
@@ -3729,10 +3729,10 @@
         <v>56</v>
       </c>
       <c r="B107" s="7">
-        <v>46049</v>
+        <v>46050</v>
       </c>
       <c r="C107" s="9" t="n">
-        <v>17.00</v>
+        <v>25.00</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>186</v>
@@ -3752,10 +3752,10 @@
         <v>56</v>
       </c>
       <c r="B108" s="7">
-        <v>46048</v>
+        <v>46049</v>
       </c>
       <c r="C108" s="9" t="n">
-        <v>8.00</v>
+        <v>17.00</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>186</v>
@@ -3772,25 +3772,25 @@
     </row>
     <row r="109" spans="1:7" ht="16.5" customHeight="1">
       <c r="A109" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B109" s="7">
-        <v>46175</v>
+        <v>46048</v>
       </c>
       <c r="C109" s="9" t="n">
-        <v>100.00</v>
+        <v>8.00</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E109" s="12" t="n">
-        <v>17960718.39</v>
+        <v>94079929.55</v>
       </c>
       <c r="F109" s="12" t="n">
-        <v>8988732.27</v>
+        <v>58829247.40</v>
       </c>
       <c r="G109" s="12" t="n">
-        <v>8971986.12</v>
+        <v>35250682.15</v>
       </c>
     </row>
     <row r="110" spans="1:7" ht="16.5" customHeight="1">
@@ -3798,10 +3798,10 @@
         <v>57</v>
       </c>
       <c r="B110" s="7">
-        <v>46153</v>
+        <v>46175</v>
       </c>
       <c r="C110" s="9" t="n">
-        <v>95.00</v>
+        <v>100.00</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>187</v>
@@ -3821,7 +3821,7 @@
         <v>57</v>
       </c>
       <c r="B111" s="7">
-        <v>46136</v>
+        <v>46153</v>
       </c>
       <c r="C111" s="9" t="n">
         <v>95.00</v>
@@ -3844,10 +3844,10 @@
         <v>57</v>
       </c>
       <c r="B112" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="C112" s="9" t="n">
-        <v>60.00</v>
+        <v>95.00</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>187</v>
@@ -3864,48 +3864,48 @@
     </row>
     <row r="113" spans="1:7" ht="16.5" customHeight="1">
       <c r="A113" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B113" s="7">
-        <v>46063</v>
+        <v>46135</v>
       </c>
       <c r="C113" s="9" t="n">
-        <v>90.00</v>
+        <v>60.00</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E113" s="12" t="n">
-        <v>508343.65</v>
+        <v>17960718.39</v>
       </c>
       <c r="F113" s="12" t="n">
-        <v>420208.91</v>
+        <v>8988732.27</v>
       </c>
       <c r="G113" s="12" t="n">
-        <v>88134.74</v>
+        <v>8971986.12</v>
       </c>
     </row>
     <row r="114" spans="1:7" ht="16.5" customHeight="1">
       <c r="A114" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B114" s="7">
-        <v>46153</v>
+        <v>46063</v>
       </c>
       <c r="C114" s="9" t="n">
-        <v>100.00</v>
+        <v>90.00</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E114" s="12" t="n">
-        <v>3583115.80</v>
+        <v>508343.65</v>
       </c>
       <c r="F114" s="12" t="n">
-        <v>3167853.46</v>
+        <v>420208.91</v>
       </c>
       <c r="G114" s="12" t="n">
-        <v>415262.34</v>
+        <v>88134.74</v>
       </c>
     </row>
     <row r="115" spans="1:7" ht="16.5" customHeight="1">
@@ -3913,10 +3913,10 @@
         <v>59</v>
       </c>
       <c r="B115" s="7">
-        <v>46139</v>
+        <v>46153</v>
       </c>
       <c r="C115" s="9" t="n">
-        <v>80.00</v>
+        <v>100.00</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>189</v>
@@ -3932,210 +3932,210 @@
       </c>
     </row>
     <row r="116" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A116" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B116" s="6">
-        <v>46146</v>
-      </c>
-      <c r="C116" s="8" t="n">
-        <v>100.00</v>
-      </c>
-      <c r="D116" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="E116" s="11" t="n">
-        <v>218199.31</v>
-      </c>
-      <c r="F116" s="11" t="n">
-        <v>588292.47</v>
-      </c>
-      <c r="G116" s="11" t="n">
-        <v>-370093.16</v>
+      <c r="A116" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B116" s="7">
+        <v>46139</v>
+      </c>
+      <c r="C116" s="9" t="n">
+        <v>80.00</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="E116" s="12" t="n">
+        <v>3583115.80</v>
+      </c>
+      <c r="F116" s="12" t="n">
+        <v>3167853.46</v>
+      </c>
+      <c r="G116" s="12" t="n">
+        <v>415262.34</v>
       </c>
     </row>
     <row r="117" spans="1:7" ht="16.5" customHeight="1">
       <c r="A117" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B117" s="6">
-        <v>46150</v>
+        <v>46146</v>
       </c>
       <c r="C117" s="8" t="n">
         <v>100.00</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E117" s="11" t="n">
-        <v>564671.38</v>
+        <v>218199.31</v>
       </c>
       <c r="F117" s="11" t="n">
-        <v>840417.82</v>
+        <v>588292.47</v>
       </c>
       <c r="G117" s="11" t="n">
-        <v>-275746.44</v>
+        <v>-370093.16</v>
       </c>
     </row>
     <row r="118" spans="1:7" ht="16.5" customHeight="1">
       <c r="A118" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B118" s="6">
-        <v>46101</v>
+        <v>46150</v>
       </c>
       <c r="C118" s="8" t="n">
-        <v>90.00</v>
+        <v>100.00</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E118" s="11" t="n">
-        <v>183494.94</v>
+        <v>564671.38</v>
       </c>
       <c r="F118" s="11" t="n">
-        <v>336167.13</v>
+        <v>840417.82</v>
       </c>
       <c r="G118" s="11" t="n">
-        <v>-152672.19</v>
+        <v>-275746.44</v>
       </c>
     </row>
     <row r="119" spans="1:7" ht="16.5" customHeight="1">
       <c r="A119" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B119" s="6">
-        <v>46111</v>
+        <v>46101</v>
       </c>
       <c r="C119" s="8" t="n">
         <v>90.00</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E119" s="11" t="n">
-        <v>121347.78</v>
+        <v>183494.94</v>
       </c>
       <c r="F119" s="11" t="n">
-        <v>840417.82</v>
+        <v>336167.13</v>
       </c>
       <c r="G119" s="11" t="n">
-        <v>-719070.04</v>
+        <v>-152672.19</v>
       </c>
     </row>
     <row r="120" spans="1:7" ht="16.5" customHeight="1">
       <c r="A120" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B120" s="6">
-        <v>46119</v>
+        <v>46111</v>
       </c>
       <c r="C120" s="8" t="n">
         <v>90.00</v>
       </c>
       <c r="D120" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="E120" s="11" t="n">
+        <v>121347.78</v>
+      </c>
+      <c r="F120" s="11" t="n">
+        <v>840417.82</v>
+      </c>
+      <c r="G120" s="11" t="n">
+        <v>-719070.04</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A121" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B121" s="6">
+        <v>46119</v>
+      </c>
+      <c r="C121" s="8" t="n">
+        <v>90.00</v>
+      </c>
+      <c r="D121" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="E120" s="11" t="n">
+      <c r="E121" s="11" t="n">
         <v>61029.83</v>
       </c>
-      <c r="F120" s="11" t="n">
+      <c r="F121" s="11" t="n">
         <v>420208.91</v>
       </c>
-      <c r="G120" s="11" t="n">
+      <c r="G121" s="11" t="n">
         <v>-359179.08</v>
       </c>
     </row>
-    <row r="121" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A121" s="3" t="s">
+    <row r="122" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A122" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B121" s="7">
+      <c r="B122" s="7">
         <v>46132</v>
       </c>
-      <c r="C121" s="9" t="n">
+      <c r="C122" s="9" t="n">
         <v>100.00</v>
       </c>
-      <c r="D121" s="3" t="s">
+      <c r="D122" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="E121" s="12" t="n">
+      <c r="E122" s="12" t="n">
         <v>1040490.23</v>
       </c>
-      <c r="F121" s="12" t="n">
+      <c r="F122" s="12" t="n">
         <v>946417.82</v>
       </c>
-      <c r="G121" s="12" t="n">
+      <c r="G122" s="12" t="n">
         <v>94072.41</v>
-      </c>
-    </row>
-    <row r="122" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A122" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B122" s="6">
-        <v>46139</v>
-      </c>
-      <c r="C122" s="8" t="n">
-        <v>100.00</v>
-      </c>
-      <c r="D122" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="E122" s="11" t="n">
-        <v>232318.79</v>
-      </c>
-      <c r="F122" s="11" t="n">
-        <v>420208.91</v>
-      </c>
-      <c r="G122" s="11" t="n">
-        <v>-187890.12</v>
       </c>
     </row>
     <row r="123" spans="1:7" ht="16.5" customHeight="1">
       <c r="A123" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B123" s="6">
-        <v>46146</v>
+        <v>46139</v>
       </c>
       <c r="C123" s="8" t="n">
         <v>100.00</v>
       </c>
       <c r="D123" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="E123" s="11" t="n">
+        <v>232318.79</v>
+      </c>
+      <c r="F123" s="11" t="n">
+        <v>420208.91</v>
+      </c>
+      <c r="G123" s="11" t="n">
+        <v>-187890.12</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A124" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B124" s="6">
+        <v>46146</v>
+      </c>
+      <c r="C124" s="8" t="n">
+        <v>100.00</v>
+      </c>
+      <c r="D124" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="E123" s="11" t="n">
+      <c r="E124" s="11" t="n">
         <v>137269.82</v>
       </c>
-      <c r="F123" s="11" t="n">
+      <c r="F124" s="11" t="n">
         <v>588292.47</v>
       </c>
-      <c r="G123" s="11" t="n">
+      <c r="G124" s="11" t="n">
         <v>-451022.65</v>
-      </c>
-    </row>
-    <row r="124" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A124" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B124" s="7">
-        <v>46146</v>
-      </c>
-      <c r="C124" s="9" t="n">
-        <v>100.00</v>
-      </c>
-      <c r="D124" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="E124" s="12" t="n">
-        <v>13145893.22</v>
-      </c>
-      <c r="F124" s="12" t="n">
-        <v>12818267.30</v>
-      </c>
-      <c r="G124" s="12" t="n">
-        <v>327625.92</v>
       </c>
     </row>
     <row r="125" spans="1:7" ht="16.5" customHeight="1">
@@ -4143,10 +4143,10 @@
         <v>68</v>
       </c>
       <c r="B125" s="7">
-        <v>46142</v>
+        <v>46146</v>
       </c>
       <c r="C125" s="9" t="n">
-        <v>90.00</v>
+        <v>100.00</v>
       </c>
       <c r="D125" s="3" t="s">
         <v>198</v>
@@ -4166,7 +4166,7 @@
         <v>68</v>
       </c>
       <c r="B126" s="7">
-        <v>46140</v>
+        <v>46142</v>
       </c>
       <c r="C126" s="9" t="n">
         <v>90.00</v>
@@ -4189,10 +4189,10 @@
         <v>68</v>
       </c>
       <c r="B127" s="7">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="C127" s="9" t="n">
-        <v>56.00</v>
+        <v>90.00</v>
       </c>
       <c r="D127" s="3" t="s">
         <v>198</v>
@@ -4212,10 +4212,10 @@
         <v>68</v>
       </c>
       <c r="B128" s="7">
-        <v>46135</v>
+        <v>46139</v>
       </c>
       <c r="C128" s="9" t="n">
-        <v>35.00</v>
+        <v>56.00</v>
       </c>
       <c r="D128" s="3" t="s">
         <v>198</v>
@@ -4235,10 +4235,10 @@
         <v>68</v>
       </c>
       <c r="B129" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="C129" s="9" t="n">
-        <v>15.00</v>
+        <v>35.00</v>
       </c>
       <c r="D129" s="3" t="s">
         <v>198</v>
@@ -4254,31 +4254,31 @@
       </c>
     </row>
     <row r="130" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A130" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B130" s="6">
-        <v>46146</v>
-      </c>
-      <c r="C130" s="8" t="n">
-        <v>100.00</v>
-      </c>
-      <c r="D130" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="E130" s="11" t="n">
-        <v>67810.92</v>
-      </c>
-      <c r="F130" s="11" t="n">
-        <v>672334.26</v>
-      </c>
-      <c r="G130" s="11" t="n">
-        <v>-604523.34</v>
+      <c r="A130" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B130" s="7">
+        <v>46134</v>
+      </c>
+      <c r="C130" s="9" t="n">
+        <v>15.00</v>
+      </c>
+      <c r="D130" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="E130" s="12" t="n">
+        <v>13145893.22</v>
+      </c>
+      <c r="F130" s="12" t="n">
+        <v>12818267.30</v>
+      </c>
+      <c r="G130" s="12" t="n">
+        <v>327625.92</v>
       </c>
     </row>
     <row r="131" spans="1:7" ht="16.5" customHeight="1">
       <c r="A131" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B131" s="6">
         <v>46146</v>
@@ -4287,85 +4287,85 @@
         <v>100.00</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E131" s="11" t="n">
-        <v>203883.27</v>
+        <v>67810.92</v>
       </c>
       <c r="F131" s="11" t="n">
         <v>672334.26</v>
       </c>
       <c r="G131" s="11" t="n">
+        <v>-604523.34</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A132" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B132" s="6">
+        <v>46146</v>
+      </c>
+      <c r="C132" s="8" t="n">
+        <v>100.00</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="E132" s="11" t="n">
+        <v>203883.27</v>
+      </c>
+      <c r="F132" s="11" t="n">
+        <v>672334.26</v>
+      </c>
+      <c r="G132" s="11" t="n">
         <v>-468450.99</v>
-      </c>
-    </row>
-    <row r="132" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A132" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="B132" s="7">
-        <v>46144</v>
-      </c>
-      <c r="C132" s="9" t="n">
-        <v>100.00</v>
-      </c>
-      <c r="D132" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="E132" s="12" t="n">
-        <v>567348.57</v>
-      </c>
-      <c r="F132" s="12" t="n">
-        <v>477000.00</v>
-      </c>
-      <c r="G132" s="12" t="n">
-        <v>90348.57</v>
       </c>
     </row>
     <row r="133" spans="1:7" ht="16.5" customHeight="1">
       <c r="A133" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B133" s="7">
-        <v>46175</v>
+        <v>46144</v>
       </c>
       <c r="C133" s="9" t="n">
         <v>100.00</v>
       </c>
       <c r="D133" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E133" s="12" t="n">
-        <v>405701.07</v>
+        <v>567348.57</v>
       </c>
       <c r="F133" s="12" t="n">
-        <v>252125.35</v>
+        <v>477000.00</v>
       </c>
       <c r="G133" s="12" t="n">
-        <v>153575.72</v>
+        <v>90348.57</v>
       </c>
     </row>
     <row r="134" spans="1:7" ht="16.5" customHeight="1">
       <c r="A134" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B134" s="7">
-        <v>46181</v>
+        <v>46175</v>
       </c>
       <c r="C134" s="9" t="n">
         <v>100.00</v>
       </c>
       <c r="D134" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E134" s="12" t="n">
-        <v>9903715.08</v>
+        <v>405701.07</v>
       </c>
       <c r="F134" s="12" t="n">
-        <v>6134306.92</v>
+        <v>252125.35</v>
       </c>
       <c r="G134" s="12" t="n">
-        <v>3769408.16</v>
+        <v>153575.72</v>
       </c>
     </row>
     <row r="135" spans="1:7" ht="16.5" customHeight="1">
@@ -4373,10 +4373,10 @@
         <v>73</v>
       </c>
       <c r="B135" s="7">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="C135" s="9" t="n">
-        <v>60.00</v>
+        <v>100.00</v>
       </c>
       <c r="D135" s="3" t="s">
         <v>203</v>
@@ -4393,25 +4393,25 @@
     </row>
     <row r="136" spans="1:7" ht="16.5" customHeight="1">
       <c r="A136" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B136" s="7">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="C136" s="9" t="n">
-        <v>100.00</v>
+        <v>60.00</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E136" s="12" t="n">
-        <v>10864319.94</v>
+        <v>9903715.08</v>
       </c>
       <c r="F136" s="12" t="n">
-        <v>6881606.92</v>
+        <v>6134306.92</v>
       </c>
       <c r="G136" s="12" t="n">
-        <v>3982713.02</v>
+        <v>3769408.16</v>
       </c>
     </row>
     <row r="137" spans="1:7" ht="16.5" customHeight="1">
@@ -4419,10 +4419,10 @@
         <v>74</v>
       </c>
       <c r="B137" s="7">
-        <v>46164</v>
+        <v>46175</v>
       </c>
       <c r="C137" s="9" t="n">
-        <v>85.00</v>
+        <v>100.00</v>
       </c>
       <c r="D137" s="3" t="s">
         <v>204</v>
@@ -4438,192 +4438,192 @@
       </c>
     </row>
     <row r="138" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A138" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B138" s="6">
-        <v>46149</v>
-      </c>
-      <c r="C138" s="8" t="n">
-        <v>100.00</v>
-      </c>
-      <c r="D138" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="E138" s="11" t="n">
-        <v>137269.82</v>
-      </c>
-      <c r="F138" s="11" t="n">
-        <v>840417.82</v>
-      </c>
-      <c r="G138" s="11" t="n">
-        <v>-703148.00</v>
+      <c r="A138" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B138" s="7">
+        <v>46164</v>
+      </c>
+      <c r="C138" s="9" t="n">
+        <v>85.00</v>
+      </c>
+      <c r="D138" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="E138" s="12" t="n">
+        <v>10864319.94</v>
+      </c>
+      <c r="F138" s="12" t="n">
+        <v>6881606.92</v>
+      </c>
+      <c r="G138" s="12" t="n">
+        <v>3982713.02</v>
       </c>
     </row>
     <row r="139" spans="1:7" ht="16.5" customHeight="1">
       <c r="A139" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B139" s="6">
-        <v>46161</v>
+        <v>46149</v>
       </c>
       <c r="C139" s="8" t="n">
         <v>100.00</v>
       </c>
       <c r="D139" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="E139" s="11" t="n">
+        <v>137269.82</v>
+      </c>
+      <c r="F139" s="11" t="n">
+        <v>840417.82</v>
+      </c>
+      <c r="G139" s="11" t="n">
+        <v>-703148.00</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A140" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B140" s="6">
+        <v>46161</v>
+      </c>
+      <c r="C140" s="8" t="n">
+        <v>100.00</v>
+      </c>
+      <c r="D140" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="E139" s="11" t="n">
+      <c r="E140" s="11" t="n">
         <v>199314.38</v>
       </c>
-      <c r="F139" s="11" t="n">
+      <c r="F140" s="11" t="n">
         <v>336167.13</v>
       </c>
-      <c r="G139" s="11" t="n">
+      <c r="G140" s="11" t="n">
         <v>-136852.75</v>
       </c>
     </row>
-    <row r="140" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A140" s="3" t="s">
+    <row r="141" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A141" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B140" s="7">
+      <c r="B141" s="7">
         <v>46174</v>
       </c>
-      <c r="C140" s="9" t="n">
+      <c r="C141" s="9" t="n">
         <v>20.00</v>
       </c>
-      <c r="D140" s="3" t="s">
+      <c r="D141" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="E140" s="12" t="n">
+      <c r="E141" s="12" t="n">
         <v>6256891.48</v>
       </c>
-      <c r="F140" s="12" t="n">
+      <c r="F141" s="12" t="n">
         <v>840417.82</v>
       </c>
-      <c r="G140" s="12" t="n">
+      <c r="G141" s="12" t="n">
         <v>5416473.66</v>
-      </c>
-    </row>
-    <row r="141" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A141" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B141" s="6">
-        <v>46174</v>
-      </c>
-      <c r="C141" s="8" t="n">
-        <v>100.00</v>
-      </c>
-      <c r="D141" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="E141" s="11" t="n">
-        <v>17285.71</v>
-      </c>
-      <c r="F141" s="11" t="n">
-        <v>252125.35</v>
-      </c>
-      <c r="G141" s="11" t="n">
-        <v>-234839.29</v>
       </c>
     </row>
     <row r="142" spans="1:7" ht="16.5" customHeight="1">
       <c r="A142" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B142" s="6">
-        <v>46161</v>
+        <v>46174</v>
       </c>
       <c r="C142" s="8" t="n">
         <v>100.00</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E142" s="11" t="n">
-        <v>203883.27</v>
+        <v>17285.71</v>
       </c>
       <c r="F142" s="11" t="n">
-        <v>336167.13</v>
+        <v>252125.35</v>
       </c>
       <c r="G142" s="11" t="n">
-        <v>-132283.86</v>
+        <v>-234839.29</v>
       </c>
     </row>
     <row r="143" spans="1:7" ht="16.5" customHeight="1">
       <c r="A143" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B143" s="6">
-        <v>46174</v>
+        <v>46161</v>
       </c>
       <c r="C143" s="8" t="n">
         <v>100.00</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E143" s="11" t="n">
         <v>203883.27</v>
       </c>
       <c r="F143" s="11" t="n">
+        <v>336167.13</v>
+      </c>
+      <c r="G143" s="11" t="n">
+        <v>-132283.86</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A144" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B144" s="6">
+        <v>46174</v>
+      </c>
+      <c r="C144" s="8" t="n">
+        <v>100.00</v>
+      </c>
+      <c r="D144" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E144" s="11" t="n">
+        <v>203883.27</v>
+      </c>
+      <c r="F144" s="11" t="n">
         <v>252125.35</v>
       </c>
-      <c r="G143" s="11" t="n">
+      <c r="G144" s="11" t="n">
         <v>-48242.08</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A144" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B144" s="7">
-        <v>46174</v>
-      </c>
-      <c r="C144" s="9" t="n">
-        <v>100.00</v>
-      </c>
-      <c r="D144" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="E144" s="12" t="n">
-        <v>925466.57</v>
-      </c>
-      <c r="F144" s="12" t="n">
-        <v>0.00</v>
-      </c>
-      <c r="G144" s="12" t="n">
-        <v>925466.57</v>
       </c>
     </row>
     <row r="145" spans="1:7" ht="16.5" customHeight="1">
       <c r="A145" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B145" s="7">
-        <v>46182</v>
+        <v>46174</v>
       </c>
       <c r="C145" s="9" t="n">
         <v>100.00</v>
       </c>
       <c r="D145" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E145" s="12" t="n">
-        <v>507687.92</v>
+        <v>925466.57</v>
       </c>
       <c r="F145" s="12" t="n">
-        <v>420208.91</v>
+        <v>0.00</v>
       </c>
       <c r="G145" s="12" t="n">
-        <v>87479.01</v>
+        <v>925466.57</v>
       </c>
     </row>
     <row r="146" spans="1:7" ht="16.5" customHeight="1">
       <c r="A146" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B146" s="7">
         <v>46182</v>
@@ -4632,85 +4632,85 @@
         <v>100.00</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E146" s="12" t="n">
-        <v>835486.55</v>
+        <v>507687.92</v>
       </c>
       <c r="F146" s="12" t="n">
         <v>420208.91</v>
       </c>
       <c r="G146" s="12" t="n">
-        <v>415277.64</v>
+        <v>87479.01</v>
       </c>
     </row>
     <row r="147" spans="1:7" ht="16.5" customHeight="1">
       <c r="A147" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B147" s="7">
-        <v>46081</v>
+        <v>46182</v>
       </c>
       <c r="C147" s="9" t="n">
         <v>100.00</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E147" s="12" t="n">
-        <v>203561619.00</v>
+        <v>835486.55</v>
       </c>
       <c r="F147" s="12" t="n">
-        <v>148320500.00</v>
+        <v>420208.91</v>
       </c>
       <c r="G147" s="12" t="n">
-        <v>55241119.00</v>
+        <v>415277.64</v>
       </c>
     </row>
     <row r="148" spans="1:7" ht="16.5" customHeight="1">
       <c r="A148" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B148" s="7">
         <v>46081</v>
       </c>
       <c r="C148" s="9" t="n">
-        <v>61.00</v>
+        <v>100.00</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E148" s="12" t="n">
-        <v>127171014.53</v>
+        <v>203561619.00</v>
       </c>
       <c r="F148" s="12" t="n">
-        <v>93283710.00</v>
+        <v>148320500.00</v>
       </c>
       <c r="G148" s="12" t="n">
-        <v>33887304.53</v>
+        <v>55241119.00</v>
       </c>
     </row>
     <row r="149" spans="1:7" ht="16.5" customHeight="1">
       <c r="A149" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B149" s="7">
-        <v>46064</v>
+        <v>46081</v>
       </c>
       <c r="C149" s="9" t="n">
-        <v>100.00</v>
+        <v>61.00</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E149" s="12" t="n">
-        <v>165630000.00</v>
+        <v>127171014.53</v>
       </c>
       <c r="F149" s="12" t="n">
-        <v>36165502.94</v>
+        <v>93283710.00</v>
       </c>
       <c r="G149" s="12" t="n">
-        <v>129464497.06</v>
+        <v>33887304.53</v>
       </c>
     </row>
     <row r="150" spans="1:7" ht="16.5" customHeight="1">
@@ -4718,7 +4718,7 @@
         <v>86</v>
       </c>
       <c r="B150" s="7">
-        <v>46063</v>
+        <v>46064</v>
       </c>
       <c r="C150" s="9" t="n">
         <v>100.00</v>
@@ -4741,7 +4741,7 @@
         <v>86</v>
       </c>
       <c r="B151" s="7">
-        <v>46062</v>
+        <v>46063</v>
       </c>
       <c r="C151" s="9" t="n">
         <v>100.00</v>
@@ -4764,10 +4764,10 @@
         <v>86</v>
       </c>
       <c r="B152" s="7">
-        <v>46060</v>
+        <v>46062</v>
       </c>
       <c r="C152" s="9" t="n">
-        <v>98.00</v>
+        <v>100.00</v>
       </c>
       <c r="D152" s="3" t="s">
         <v>216</v>
@@ -4787,10 +4787,10 @@
         <v>86</v>
       </c>
       <c r="B153" s="7">
-        <v>46059</v>
+        <v>46060</v>
       </c>
       <c r="C153" s="9" t="n">
-        <v>96.00</v>
+        <v>98.00</v>
       </c>
       <c r="D153" s="3" t="s">
         <v>216</v>
@@ -4810,10 +4810,10 @@
         <v>86</v>
       </c>
       <c r="B154" s="7">
-        <v>46058</v>
+        <v>46059</v>
       </c>
       <c r="C154" s="9" t="n">
-        <v>92.00</v>
+        <v>96.00</v>
       </c>
       <c r="D154" s="3" t="s">
         <v>216</v>
@@ -4833,10 +4833,10 @@
         <v>86</v>
       </c>
       <c r="B155" s="7">
-        <v>46057</v>
+        <v>46058</v>
       </c>
       <c r="C155" s="9" t="n">
-        <v>87.00</v>
+        <v>92.00</v>
       </c>
       <c r="D155" s="3" t="s">
         <v>216</v>
@@ -4856,10 +4856,10 @@
         <v>86</v>
       </c>
       <c r="B156" s="7">
-        <v>46055</v>
+        <v>46057</v>
       </c>
       <c r="C156" s="9" t="n">
-        <v>78.00</v>
+        <v>87.00</v>
       </c>
       <c r="D156" s="3" t="s">
         <v>216</v>
@@ -4879,10 +4879,10 @@
         <v>86</v>
       </c>
       <c r="B157" s="7">
-        <v>46053</v>
+        <v>46055</v>
       </c>
       <c r="C157" s="9" t="n">
-        <v>73.00</v>
+        <v>78.00</v>
       </c>
       <c r="D157" s="3" t="s">
         <v>216</v>
@@ -4902,10 +4902,10 @@
         <v>86</v>
       </c>
       <c r="B158" s="7">
-        <v>46052</v>
+        <v>46053</v>
       </c>
       <c r="C158" s="9" t="n">
-        <v>66.00</v>
+        <v>73.00</v>
       </c>
       <c r="D158" s="3" t="s">
         <v>216</v>
@@ -4925,10 +4925,10 @@
         <v>86</v>
       </c>
       <c r="B159" s="7">
-        <v>46051</v>
+        <v>46052</v>
       </c>
       <c r="C159" s="9" t="n">
-        <v>61.00</v>
+        <v>66.00</v>
       </c>
       <c r="D159" s="3" t="s">
         <v>216</v>
@@ -4948,10 +4948,10 @@
         <v>86</v>
       </c>
       <c r="B160" s="7">
-        <v>46050</v>
+        <v>46051</v>
       </c>
       <c r="C160" s="9" t="n">
-        <v>59.00</v>
+        <v>61.00</v>
       </c>
       <c r="D160" s="3" t="s">
         <v>216</v>
@@ -4971,10 +4971,10 @@
         <v>86</v>
       </c>
       <c r="B161" s="7">
-        <v>46049</v>
+        <v>46050</v>
       </c>
       <c r="C161" s="9" t="n">
-        <v>56.00</v>
+        <v>59.00</v>
       </c>
       <c r="D161" s="3" t="s">
         <v>216</v>
@@ -4994,10 +4994,10 @@
         <v>86</v>
       </c>
       <c r="B162" s="7">
-        <v>46048</v>
+        <v>46049</v>
       </c>
       <c r="C162" s="9" t="n">
-        <v>50.00</v>
+        <v>56.00</v>
       </c>
       <c r="D162" s="3" t="s">
         <v>216</v>
@@ -5017,10 +5017,10 @@
         <v>86</v>
       </c>
       <c r="B163" s="7">
-        <v>46047</v>
+        <v>46048</v>
       </c>
       <c r="C163" s="9" t="n">
-        <v>36.00</v>
+        <v>50.00</v>
       </c>
       <c r="D163" s="3" t="s">
         <v>216</v>
@@ -5040,10 +5040,10 @@
         <v>86</v>
       </c>
       <c r="B164" s="7">
-        <v>46046</v>
+        <v>46047</v>
       </c>
       <c r="C164" s="9" t="n">
-        <v>20.00</v>
+        <v>36.00</v>
       </c>
       <c r="D164" s="3" t="s">
         <v>216</v>
@@ -5063,10 +5063,10 @@
         <v>86</v>
       </c>
       <c r="B165" s="7">
-        <v>46026</v>
+        <v>46046</v>
       </c>
       <c r="C165" s="9" t="n">
-        <v>14.00</v>
+        <v>20.00</v>
       </c>
       <c r="D165" s="3" t="s">
         <v>216</v>
@@ -5086,10 +5086,10 @@
         <v>86</v>
       </c>
       <c r="B166" s="7">
-        <v>46025</v>
+        <v>46026</v>
       </c>
       <c r="C166" s="9" t="n">
-        <v>10.00</v>
+        <v>14.00</v>
       </c>
       <c r="D166" s="3" t="s">
         <v>216</v>
@@ -5109,10 +5109,10 @@
         <v>86</v>
       </c>
       <c r="B167" s="7">
-        <v>46024</v>
+        <v>46025</v>
       </c>
       <c r="C167" s="9" t="n">
-        <v>5.00</v>
+        <v>10.00</v>
       </c>
       <c r="D167" s="3" t="s">
         <v>216</v>
@@ -5129,25 +5129,25 @@
     </row>
     <row r="168" spans="1:7" ht="16.5" customHeight="1">
       <c r="A168" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B168" s="7">
-        <v>46077</v>
+        <v>46024</v>
       </c>
       <c r="C168" s="9" t="n">
-        <v>100.00</v>
+        <v>5.00</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E168" s="12" t="n">
-        <v>3784091.75</v>
+        <v>165630000.00</v>
       </c>
       <c r="F168" s="12" t="n">
-        <v>2073035.64</v>
+        <v>36165502.94</v>
       </c>
       <c r="G168" s="12" t="n">
-        <v>1711055.75</v>
+        <v>129464497.06</v>
       </c>
     </row>
     <row r="169" spans="1:7" ht="16.5" customHeight="1">
@@ -5155,10 +5155,10 @@
         <v>87</v>
       </c>
       <c r="B169" s="7">
-        <v>46076</v>
+        <v>46077</v>
       </c>
       <c r="C169" s="9" t="n">
-        <v>98.00</v>
+        <v>100.00</v>
       </c>
       <c r="D169" s="3" t="s">
         <v>217</v>
@@ -5178,10 +5178,10 @@
         <v>87</v>
       </c>
       <c r="B170" s="7">
-        <v>46064</v>
+        <v>46076</v>
       </c>
       <c r="C170" s="9" t="n">
-        <v>37.00</v>
+        <v>98.00</v>
       </c>
       <c r="D170" s="3" t="s">
         <v>217</v>
@@ -5198,94 +5198,94 @@
     </row>
     <row r="171" spans="1:7" ht="16.5" customHeight="1">
       <c r="A171" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B171" s="7">
-        <v>46091</v>
+        <v>46064</v>
       </c>
       <c r="C171" s="9" t="n">
-        <v>100.00</v>
+        <v>37.00</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E171" s="12" t="n">
-        <v>18500000.00</v>
+        <v>3784091.75</v>
       </c>
       <c r="F171" s="12" t="n">
-        <v>17329453.46</v>
+        <v>2073035.64</v>
       </c>
       <c r="G171" s="12" t="n">
-        <v>1170546.54</v>
+        <v>1711055.75</v>
       </c>
     </row>
     <row r="172" spans="1:7" ht="16.5" customHeight="1">
       <c r="A172" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B172" s="7">
-        <v>46073</v>
+        <v>46091</v>
       </c>
       <c r="C172" s="9" t="n">
-        <v>50.00</v>
+        <v>100.00</v>
       </c>
       <c r="D172" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E172" s="12" t="n">
-        <v>2076372.55</v>
+        <v>18500000.00</v>
       </c>
       <c r="F172" s="12" t="n">
-        <v>840417.82</v>
+        <v>17329453.46</v>
       </c>
       <c r="G172" s="12" t="n">
-        <v>1235954.73</v>
+        <v>1170546.54</v>
       </c>
     </row>
     <row r="173" spans="1:7" ht="16.5" customHeight="1">
       <c r="A173" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B173" s="7">
-        <v>46037</v>
+        <v>46073</v>
       </c>
       <c r="C173" s="9" t="n">
-        <v>25.00</v>
+        <v>50.00</v>
       </c>
       <c r="D173" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E173" s="12" t="n">
-        <v>5515126.23</v>
+        <v>2076372.55</v>
       </c>
       <c r="F173" s="12" t="n">
-        <v>1260626.73</v>
+        <v>840417.82</v>
       </c>
       <c r="G173" s="12" t="n">
-        <v>4254499.50</v>
+        <v>1235954.73</v>
       </c>
     </row>
     <row r="174" spans="1:7" ht="16.5" customHeight="1">
       <c r="A174" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B174" s="7">
-        <v>46115</v>
+        <v>46037</v>
       </c>
       <c r="C174" s="9" t="n">
-        <v>70.00</v>
+        <v>25.00</v>
       </c>
       <c r="D174" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E174" s="12" t="n">
-        <v>5582787.78</v>
+        <v>5515126.23</v>
       </c>
       <c r="F174" s="12" t="n">
-        <v>3467671.28</v>
+        <v>1260626.73</v>
       </c>
       <c r="G174" s="12" t="n">
-        <v>2115116.50</v>
+        <v>4254499.50</v>
       </c>
     </row>
     <row r="175" spans="1:7" ht="16.5" customHeight="1">
@@ -5293,10 +5293,10 @@
         <v>91</v>
       </c>
       <c r="B175" s="7">
-        <v>45722</v>
+        <v>46115</v>
       </c>
       <c r="C175" s="9" t="n">
-        <v>40.00</v>
+        <v>70.00</v>
       </c>
       <c r="D175" s="3" t="s">
         <v>221</v>
@@ -5313,48 +5313,48 @@
     </row>
     <row r="176" spans="1:7" ht="16.5" customHeight="1">
       <c r="A176" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B176" s="7">
-        <v>45971</v>
+        <v>45722</v>
       </c>
       <c r="C176" s="9" t="n">
-        <v>100.00</v>
+        <v>40.00</v>
       </c>
       <c r="D176" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E176" s="12" t="n">
-        <v>29094323.80</v>
+        <v>5582787.78</v>
       </c>
       <c r="F176" s="12" t="n">
-        <v>15984649.48</v>
+        <v>3467671.28</v>
       </c>
       <c r="G176" s="12" t="n">
-        <v>13109674.32</v>
+        <v>2115116.50</v>
       </c>
     </row>
     <row r="177" spans="1:7" ht="16.5" customHeight="1">
       <c r="A177" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B177" s="7">
-        <v>46078</v>
+        <v>45971</v>
       </c>
       <c r="C177" s="9" t="n">
         <v>100.00</v>
       </c>
       <c r="D177" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E177" s="12" t="n">
-        <v>9730904.60</v>
+        <v>29094323.80</v>
       </c>
       <c r="F177" s="12" t="n">
-        <v>4202089.10</v>
+        <v>15984649.48</v>
       </c>
       <c r="G177" s="12" t="n">
-        <v>5528815.50</v>
+        <v>13109674.32</v>
       </c>
     </row>
     <row r="178" spans="1:7" ht="16.5" customHeight="1">
@@ -5362,10 +5362,10 @@
         <v>93</v>
       </c>
       <c r="B178" s="7">
-        <v>46073</v>
+        <v>46078</v>
       </c>
       <c r="C178" s="9" t="n">
-        <v>67.00</v>
+        <v>100.00</v>
       </c>
       <c r="D178" s="3" t="s">
         <v>223</v>
@@ -5385,10 +5385,10 @@
         <v>93</v>
       </c>
       <c r="B179" s="7">
-        <v>46028</v>
+        <v>46073</v>
       </c>
       <c r="C179" s="9" t="n">
-        <v>26.00</v>
+        <v>67.00</v>
       </c>
       <c r="D179" s="3" t="s">
         <v>223</v>
@@ -5405,301 +5405,301 @@
     </row>
     <row r="180" spans="1:7" ht="16.5" customHeight="1">
       <c r="A180" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B180" s="7">
-        <v>46104</v>
+        <v>46028</v>
       </c>
       <c r="C180" s="9" t="n">
-        <v>90.00</v>
+        <v>26.00</v>
       </c>
       <c r="D180" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E180" s="12" t="n">
-        <v>4960679.95</v>
+        <v>9730904.60</v>
       </c>
       <c r="F180" s="12" t="n">
-        <v>4869889.10</v>
+        <v>4202089.10</v>
       </c>
       <c r="G180" s="12" t="n">
-        <v>90790.95</v>
+        <v>5528815.50</v>
       </c>
     </row>
     <row r="181" spans="1:7" ht="16.5" customHeight="1">
       <c r="A181" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B181" s="7">
-        <v>45994</v>
+        <v>46104</v>
       </c>
       <c r="C181" s="9" t="n">
-        <v>100.00</v>
+        <v>90.00</v>
       </c>
       <c r="D181" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E181" s="12" t="n">
-        <v>13265457.76</v>
+        <v>4960679.95</v>
       </c>
       <c r="F181" s="12" t="n">
-        <v>8426924.74</v>
+        <v>4869889.10</v>
       </c>
       <c r="G181" s="12" t="n">
-        <v>4838532.76</v>
+        <v>90790.95</v>
       </c>
     </row>
     <row r="182" spans="1:7" ht="16.5" customHeight="1">
       <c r="A182" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B182" s="7">
-        <v>45986</v>
+        <v>45994</v>
       </c>
       <c r="C182" s="9" t="n">
-        <v>30.00</v>
+        <v>100.00</v>
       </c>
       <c r="D182" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E182" s="12" t="n">
-        <v>23873307.57</v>
+        <v>13265457.76</v>
       </c>
       <c r="F182" s="12" t="n">
-        <v>8504142.56</v>
+        <v>8426924.74</v>
       </c>
       <c r="G182" s="12" t="n">
-        <v>15369165.01</v>
+        <v>4838532.76</v>
       </c>
     </row>
     <row r="183" spans="1:7" ht="16.5" customHeight="1">
       <c r="A183" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B183" s="7">
-        <v>46028</v>
+        <v>45986</v>
       </c>
       <c r="C183" s="9" t="n">
-        <v>90.00</v>
+        <v>30.00</v>
       </c>
       <c r="D183" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E183" s="12" t="n">
-        <v>22888437.30</v>
+        <v>23873307.57</v>
       </c>
       <c r="F183" s="12" t="n">
-        <v>8716142.56</v>
+        <v>8504142.56</v>
       </c>
       <c r="G183" s="12" t="n">
-        <v>14172294.74</v>
+        <v>15369165.01</v>
       </c>
     </row>
     <row r="184" spans="1:7" ht="16.5" customHeight="1">
       <c r="A184" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B184" s="7">
+        <v>46028</v>
+      </c>
+      <c r="C184" s="9" t="n">
+        <v>90.00</v>
+      </c>
+      <c r="D184" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="E184" s="12" t="n">
+        <v>22888437.30</v>
+      </c>
+      <c r="F184" s="12" t="n">
+        <v>8716142.56</v>
+      </c>
+      <c r="G184" s="12" t="n">
+        <v>14172294.74</v>
+      </c>
+    </row>
+    <row r="185" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A185" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B184" s="7">
+      <c r="B185" s="7">
         <v>46057</v>
       </c>
-      <c r="C184" s="9" t="n">
+      <c r="C185" s="9" t="n">
         <v>95.00</v>
       </c>
-      <c r="D184" s="3" t="s">
+      <c r="D185" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="E184" s="12" t="n">
+      <c r="E185" s="12" t="n">
         <v>847087.63</v>
       </c>
-      <c r="F184" s="12" t="n">
+      <c r="F185" s="12" t="n">
         <v>840417.82</v>
       </c>
-      <c r="G184" s="12" t="n">
+      <c r="G185" s="12" t="n">
         <v>6669.63</v>
-      </c>
-    </row>
-    <row r="185" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A185" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B185" s="6">
-        <v>46181</v>
-      </c>
-      <c r="C185" s="8" t="n">
-        <v>100.00</v>
-      </c>
-      <c r="D185" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="E185" s="11" t="n">
-        <v>1131124.74</v>
-      </c>
-      <c r="F185" s="11" t="n">
-        <v>1260626.73</v>
-      </c>
-      <c r="G185" s="11" t="n">
-        <v>-129501.99</v>
       </c>
     </row>
     <row r="186" spans="1:7" ht="16.5" customHeight="1">
       <c r="A186" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B186" s="6">
+        <v>46181</v>
+      </c>
+      <c r="C186" s="8" t="n">
+        <v>100.00</v>
+      </c>
+      <c r="D186" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="E186" s="11" t="n">
+        <v>1131124.74</v>
+      </c>
+      <c r="F186" s="11" t="n">
+        <v>1260626.73</v>
+      </c>
+      <c r="G186" s="11" t="n">
+        <v>-129501.99</v>
+      </c>
+    </row>
+    <row r="187" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A187" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B186" s="6">
+      <c r="B187" s="6">
         <v>46168</v>
       </c>
-      <c r="C186" s="8" t="n">
+      <c r="C187" s="8" t="n">
         <v>14.00</v>
       </c>
-      <c r="D186" s="2" t="s">
+      <c r="D187" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="E186" s="11" t="n">
+      <c r="E187" s="11" t="n">
         <v>2425416.39</v>
       </c>
-      <c r="F186" s="11" t="n">
+      <c r="F187" s="11" t="n">
         <v>3361671.28</v>
       </c>
-      <c r="G186" s="11" t="n">
+      <c r="G187" s="11" t="n">
         <v>-936254.89</v>
       </c>
     </row>
-    <row r="187" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A187" s="3" t="s">
+    <row r="188" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A188" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="B187" s="7">
+      <c r="B188" s="7">
         <v>46084</v>
       </c>
-      <c r="C187" s="9" t="n">
+      <c r="C188" s="9" t="n">
         <v>100.00</v>
       </c>
-      <c r="D187" s="3" t="s">
+      <c r="D188" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="E187" s="12" t="n">
+      <c r="E188" s="12" t="n">
         <v>2987518.24</v>
       </c>
-      <c r="F187" s="12" t="n">
+      <c r="F188" s="12" t="n">
         <v>1260626.73</v>
       </c>
-      <c r="G187" s="12" t="n">
+      <c r="G188" s="12" t="n">
         <v>1726891.24</v>
       </c>
     </row>
-    <row r="188" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A188" s="2" t="s">
+    <row r="189" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A189" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B188" s="6">
+      <c r="B189" s="6">
         <v>46035</v>
       </c>
-      <c r="C188" s="8" t="n">
+      <c r="C189" s="8" t="n">
         <v>100.00</v>
       </c>
-      <c r="D188" s="2" t="s">
+      <c r="D189" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="E188" s="11" t="n">
+      <c r="E189" s="11" t="n">
         <v>768952.28</v>
       </c>
-      <c r="F188" s="11" t="n">
+      <c r="F189" s="11" t="n">
         <v>1680835.64</v>
       </c>
-      <c r="G188" s="11" t="n">
+      <c r="G189" s="11" t="n">
         <v>-911883.36</v>
       </c>
     </row>
-    <row r="189" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A189" s="3" t="s">
+    <row r="190" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A190" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B189" s="7">
+      <c r="B190" s="7">
         <v>46180</v>
       </c>
-      <c r="C189" s="9" t="n">
+      <c r="C190" s="9" t="n">
         <v>100.00</v>
       </c>
-      <c r="D189" s="3" t="s">
+      <c r="D190" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="E189" s="12" t="n">
+      <c r="E190" s="12" t="n">
         <v>2459264.77</v>
       </c>
-      <c r="F189" s="12" t="n">
+      <c r="F190" s="12" t="n">
         <v>1260626.73</v>
       </c>
-      <c r="G189" s="12" t="n">
+      <c r="G190" s="12" t="n">
         <v>1198638.04</v>
       </c>
     </row>
-    <row r="190" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A190" s="2" t="s">
+    <row r="191" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A191" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B190" s="6">
+      <c r="B191" s="6">
         <v>46174</v>
       </c>
-      <c r="C190" s="8" t="n">
+      <c r="C191" s="8" t="n">
         <v>100.00</v>
       </c>
-      <c r="D190" s="2" t="s">
+      <c r="D191" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="E190" s="11" t="n">
+      <c r="E191" s="11" t="n">
         <v>279805.16</v>
       </c>
-      <c r="F190" s="11" t="n">
+      <c r="F191" s="11" t="n">
         <v>420208.91</v>
       </c>
-      <c r="G190" s="11" t="n">
+      <c r="G191" s="11" t="n">
         <v>-140403.75</v>
-      </c>
-    </row>
-    <row r="191" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A191" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B191" s="7">
-        <v>46086</v>
-      </c>
-      <c r="C191" s="9" t="n">
-        <v>30.00</v>
-      </c>
-      <c r="D191" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="E191" s="12" t="n">
-        <v>1371505.80</v>
-      </c>
-      <c r="F191" s="12" t="n">
-        <v>1260626.73</v>
-      </c>
-      <c r="G191" s="12" t="n">
-        <v>110879.07</v>
       </c>
     </row>
     <row r="192" spans="1:7" ht="16.5" customHeight="1">
       <c r="A192" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B192" s="7">
-        <v>46180</v>
+        <v>46086</v>
       </c>
       <c r="C192" s="9" t="n">
-        <v>100.00</v>
+        <v>30.00</v>
       </c>
       <c r="D192" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E192" s="12" t="n">
-        <v>4264844.14</v>
+        <v>1371505.80</v>
       </c>
       <c r="F192" s="12" t="n">
-        <v>3361671.28</v>
+        <v>1260626.73</v>
       </c>
       <c r="G192" s="12" t="n">
-        <v>903172.86</v>
+        <v>110879.07</v>
       </c>
     </row>
     <row r="193" spans="1:7" ht="16.5" customHeight="1">
@@ -5707,10 +5707,10 @@
         <v>106</v>
       </c>
       <c r="B193" s="7">
-        <v>46126</v>
+        <v>46180</v>
       </c>
       <c r="C193" s="9" t="n">
-        <v>60.00</v>
+        <v>100.00</v>
       </c>
       <c r="D193" s="3" t="s">
         <v>236</v>
@@ -5730,10 +5730,10 @@
         <v>106</v>
       </c>
       <c r="B194" s="7">
-        <v>46085</v>
+        <v>46126</v>
       </c>
       <c r="C194" s="9" t="n">
-        <v>50.00</v>
+        <v>60.00</v>
       </c>
       <c r="D194" s="3" t="s">
         <v>236</v>
@@ -5750,71 +5750,71 @@
     </row>
     <row r="195" spans="1:7" ht="16.5" customHeight="1">
       <c r="A195" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B195" s="7">
+        <v>46085</v>
+      </c>
+      <c r="C195" s="9" t="n">
+        <v>50.00</v>
+      </c>
+      <c r="D195" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="E195" s="12" t="n">
+        <v>4264844.14</v>
+      </c>
+      <c r="F195" s="12" t="n">
+        <v>3361671.28</v>
+      </c>
+      <c r="G195" s="12" t="n">
+        <v>903172.86</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A196" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="B195" s="7">
+      <c r="B196" s="7">
         <v>46028</v>
       </c>
-      <c r="C195" s="9" t="n">
+      <c r="C196" s="9" t="n">
         <v>100.00</v>
       </c>
-      <c r="D195" s="3" t="s">
+      <c r="D196" s="3" t="s">
         <v>237</v>
       </c>
-      <c r="E195" s="12" t="n">
+      <c r="E196" s="12" t="n">
         <v>1329021.15</v>
       </c>
-      <c r="F195" s="12" t="n">
+      <c r="F196" s="12" t="n">
         <v>840417.82</v>
       </c>
-      <c r="G195" s="12" t="n">
+      <c r="G196" s="12" t="n">
         <v>488603.33</v>
       </c>
     </row>
-    <row r="196" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A196" s="2" t="s">
+    <row r="197" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A197" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B196" s="6">
+      <c r="B197" s="6">
         <v>46098</v>
       </c>
-      <c r="C196" s="8" t="n">
+      <c r="C197" s="8" t="n">
         <v>100.00</v>
       </c>
-      <c r="D196" s="2" t="s">
+      <c r="D197" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="E196" s="11" t="n">
+      <c r="E197" s="11" t="n">
         <v>32195587.93</v>
       </c>
-      <c r="F196" s="11">
+      <c r="F197" s="11">
         <v/>
       </c>
-      <c r="G196" s="11">
+      <c r="G197" s="11">
         <v/>
-      </c>
-    </row>
-    <row r="197" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A197" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B197" s="7">
-        <v>46132</v>
-      </c>
-      <c r="C197" s="9" t="n">
-        <v>30.00</v>
-      </c>
-      <c r="D197" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="E197" s="12" t="n">
-        <v>8277057.96</v>
-      </c>
-      <c r="F197" s="12" t="n">
-        <v>7778042.56</v>
-      </c>
-      <c r="G197" s="12" t="n">
-        <v>499015.40</v>
       </c>
     </row>
     <row r="198" spans="1:7" ht="16.5" customHeight="1">
@@ -5822,10 +5822,10 @@
         <v>109</v>
       </c>
       <c r="B198" s="7">
-        <v>45952</v>
+        <v>46132</v>
       </c>
       <c r="C198" s="9" t="n">
-        <v>20.00</v>
+        <v>30.00</v>
       </c>
       <c r="D198" s="3" t="s">
         <v>239</v>
@@ -5841,49 +5841,49 @@
       </c>
     </row>
     <row r="199" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A199" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="B199" s="6">
-        <v>46079</v>
-      </c>
-      <c r="C199" s="8" t="n">
-        <v>100.00</v>
-      </c>
-      <c r="D199" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="E199" s="11" t="n">
-        <v>6277413.55</v>
-      </c>
-      <c r="F199" s="11" t="n">
-        <v>0.00</v>
-      </c>
-      <c r="G199" s="11">
-        <v/>
+      <c r="A199" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B199" s="7">
+        <v>45952</v>
+      </c>
+      <c r="C199" s="9" t="n">
+        <v>20.00</v>
+      </c>
+      <c r="D199" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="E199" s="12" t="n">
+        <v>8277057.96</v>
+      </c>
+      <c r="F199" s="12" t="n">
+        <v>7778042.56</v>
+      </c>
+      <c r="G199" s="12" t="n">
+        <v>499015.40</v>
       </c>
     </row>
     <row r="200" spans="1:7" ht="16.5" customHeight="1">
       <c r="A200" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B200" s="6">
-        <v>46161</v>
+        <v>46079</v>
       </c>
       <c r="C200" s="8" t="n">
-        <v>30.00</v>
+        <v>100.00</v>
       </c>
       <c r="D200" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E200" s="11" t="n">
-        <v>4268792.84</v>
+        <v>6277413.55</v>
       </c>
       <c r="F200" s="11" t="n">
-        <v>8482942.56</v>
-      </c>
-      <c r="G200" s="11" t="n">
-        <v>-4214149.73</v>
+        <v>0.00</v>
+      </c>
+      <c r="G200" s="11">
+        <v/>
       </c>
     </row>
     <row r="201" spans="1:7" ht="16.5" customHeight="1">
@@ -5891,10 +5891,10 @@
         <v>111</v>
       </c>
       <c r="B201" s="6">
-        <v>46090</v>
-      </c>
-      <c r="C201" s="8">
-        <v/>
+        <v>46161</v>
+      </c>
+      <c r="C201" s="8" t="n">
+        <v>30.00</v>
       </c>
       <c r="D201" s="2" t="s">
         <v>241</v>
@@ -5911,25 +5911,25 @@
     </row>
     <row r="202" spans="1:7" ht="16.5" customHeight="1">
       <c r="A202" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B202" s="6">
-        <v>46036</v>
-      </c>
-      <c r="C202" s="8" t="n">
-        <v>95.00</v>
+        <v>46090</v>
+      </c>
+      <c r="C202" s="8">
+        <v/>
       </c>
       <c r="D202" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E202" s="11" t="n">
-        <v>19218262.50</v>
+        <v>4268792.84</v>
       </c>
       <c r="F202" s="11" t="n">
-        <v>19291038.58</v>
+        <v>8482942.56</v>
       </c>
       <c r="G202" s="11" t="n">
-        <v>-72776.50</v>
+        <v>-4214149.73</v>
       </c>
     </row>
     <row r="203" spans="1:7" ht="16.5" customHeight="1">
@@ -5937,10 +5937,10 @@
         <v>112</v>
       </c>
       <c r="B203" s="6">
-        <v>46035</v>
+        <v>46036</v>
       </c>
       <c r="C203" s="8" t="n">
-        <v>70.00</v>
+        <v>95.00</v>
       </c>
       <c r="D203" s="2" t="s">
         <v>242</v>
@@ -5960,10 +5960,10 @@
         <v>112</v>
       </c>
       <c r="B204" s="6">
-        <v>46034</v>
+        <v>46035</v>
       </c>
       <c r="C204" s="8" t="n">
-        <v>35.00</v>
+        <v>70.00</v>
       </c>
       <c r="D204" s="2" t="s">
         <v>242</v>
@@ -5980,71 +5980,71 @@
     </row>
     <row r="205" spans="1:7" ht="16.5" customHeight="1">
       <c r="A205" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B205" s="6">
+        <v>46034</v>
+      </c>
+      <c r="C205" s="8" t="n">
+        <v>35.00</v>
+      </c>
+      <c r="D205" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="E205" s="11" t="n">
+        <v>19218262.50</v>
+      </c>
+      <c r="F205" s="11" t="n">
+        <v>19291038.58</v>
+      </c>
+      <c r="G205" s="11" t="n">
+        <v>-72776.50</v>
+      </c>
+    </row>
+    <row r="206" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A206" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B205" s="6">
+      <c r="B206" s="6">
         <v>46097</v>
       </c>
-      <c r="C205" s="8" t="n">
+      <c r="C206" s="8" t="n">
         <v>100.00</v>
       </c>
-      <c r="D205" s="2" t="s">
+      <c r="D206" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="E205" s="11" t="n">
+      <c r="E206" s="11" t="n">
         <v>5523599.87</v>
       </c>
-      <c r="F205" s="11">
+      <c r="F206" s="11">
         <v/>
       </c>
-      <c r="G205" s="11">
+      <c r="G206" s="11">
         <v/>
-      </c>
-    </row>
-    <row r="206" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A206" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="B206" s="7">
-        <v>46047</v>
-      </c>
-      <c r="C206" s="9" t="n">
-        <v>90.00</v>
-      </c>
-      <c r="D206" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="E206" s="12" t="n">
-        <v>1729369.40</v>
-      </c>
-      <c r="F206" s="12" t="n">
-        <v>840417.82</v>
-      </c>
-      <c r="G206" s="12" t="n">
-        <v>888951.40</v>
       </c>
     </row>
     <row r="207" spans="1:7" ht="16.5" customHeight="1">
       <c r="A207" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B207" s="7">
-        <v>46182</v>
+        <v>46047</v>
       </c>
       <c r="C207" s="9" t="n">
-        <v>40.00</v>
+        <v>90.00</v>
       </c>
       <c r="D207" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E207" s="12" t="n">
-        <v>15742398.24</v>
+        <v>1729369.40</v>
       </c>
       <c r="F207" s="12" t="n">
-        <v>5586898.01</v>
+        <v>840417.82</v>
       </c>
       <c r="G207" s="12" t="n">
-        <v>10155500.23</v>
+        <v>888951.40</v>
       </c>
     </row>
     <row r="208" spans="1:7" ht="16.5" customHeight="1">
@@ -6052,22 +6052,22 @@
         <v>115</v>
       </c>
       <c r="B208" s="7">
-        <v>46178</v>
+        <v>46185</v>
       </c>
       <c r="C208" s="9" t="n">
-        <v>32.00</v>
+        <v>44.00</v>
       </c>
       <c r="D208" s="3" t="s">
         <v>245</v>
       </c>
       <c r="E208" s="12" t="n">
-        <v>15742398.24</v>
+        <v>17316638.07</v>
       </c>
       <c r="F208" s="12" t="n">
-        <v>5586898.01</v>
+        <v>9404369.29</v>
       </c>
       <c r="G208" s="12" t="n">
-        <v>10155500.23</v>
+        <v>7912268.78</v>
       </c>
     </row>
     <row r="209" spans="1:7" ht="16.5" customHeight="1">
@@ -6075,68 +6075,68 @@
         <v>115</v>
       </c>
       <c r="B209" s="7">
-        <v>46155</v>
+        <v>46182</v>
       </c>
       <c r="C209" s="9" t="n">
-        <v>6.00</v>
+        <v>40.00</v>
       </c>
       <c r="D209" s="3" t="s">
         <v>245</v>
       </c>
       <c r="E209" s="12" t="n">
-        <v>15742398.24</v>
+        <v>17316638.07</v>
       </c>
       <c r="F209" s="12" t="n">
-        <v>5586898.01</v>
+        <v>9404369.29</v>
       </c>
       <c r="G209" s="12" t="n">
-        <v>10155500.23</v>
+        <v>7912268.78</v>
       </c>
     </row>
     <row r="210" spans="1:7" ht="16.5" customHeight="1">
       <c r="A210" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B210" s="7">
-        <v>46128</v>
+        <v>46178</v>
       </c>
       <c r="C210" s="9" t="n">
-        <v>100.00</v>
+        <v>32.00</v>
       </c>
       <c r="D210" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E210" s="12" t="n">
-        <v>31485245.74</v>
+        <v>17316638.07</v>
       </c>
       <c r="F210" s="12" t="n">
-        <v>17446676.21</v>
+        <v>9404369.29</v>
       </c>
       <c r="G210" s="12" t="n">
-        <v>14038569.74</v>
+        <v>7912268.78</v>
       </c>
     </row>
     <row r="211" spans="1:7" ht="16.5" customHeight="1">
       <c r="A211" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B211" s="7">
-        <v>46125</v>
+        <v>46155</v>
       </c>
       <c r="C211" s="9" t="n">
-        <v>80.00</v>
+        <v>6.00</v>
       </c>
       <c r="D211" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E211" s="12" t="n">
-        <v>31485245.74</v>
+        <v>17316638.07</v>
       </c>
       <c r="F211" s="12" t="n">
-        <v>17446676.21</v>
+        <v>9404369.29</v>
       </c>
       <c r="G211" s="12" t="n">
-        <v>14038569.74</v>
+        <v>7912268.78</v>
       </c>
     </row>
     <row r="212" spans="1:7" ht="16.5" customHeight="1">
@@ -6144,10 +6144,10 @@
         <v>116</v>
       </c>
       <c r="B212" s="7">
-        <v>46119</v>
+        <v>46128</v>
       </c>
       <c r="C212" s="9" t="n">
-        <v>54.00</v>
+        <v>100.00</v>
       </c>
       <c r="D212" s="3" t="s">
         <v>246</v>
@@ -6167,10 +6167,10 @@
         <v>116</v>
       </c>
       <c r="B213" s="7">
-        <v>46118</v>
+        <v>46125</v>
       </c>
       <c r="C213" s="9" t="n">
-        <v>52.00</v>
+        <v>80.00</v>
       </c>
       <c r="D213" s="3" t="s">
         <v>246</v>
@@ -6190,10 +6190,10 @@
         <v>116</v>
       </c>
       <c r="B214" s="7">
-        <v>46114</v>
+        <v>46119</v>
       </c>
       <c r="C214" s="9" t="n">
-        <v>35.00</v>
+        <v>54.00</v>
       </c>
       <c r="D214" s="3" t="s">
         <v>246</v>
@@ -6213,10 +6213,10 @@
         <v>116</v>
       </c>
       <c r="B215" s="7">
-        <v>46113</v>
+        <v>46118</v>
       </c>
       <c r="C215" s="9" t="n">
-        <v>35.00</v>
+        <v>52.00</v>
       </c>
       <c r="D215" s="3" t="s">
         <v>246</v>
@@ -6233,232 +6233,232 @@
     </row>
     <row r="216" spans="1:7" ht="16.5" customHeight="1">
       <c r="A216" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B216" s="7">
-        <v>46100</v>
+        <v>46114</v>
       </c>
       <c r="C216" s="9" t="n">
-        <v>75.00</v>
+        <v>35.00</v>
       </c>
       <c r="D216" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E216" s="12" t="n">
-        <v>36111431.42</v>
+        <v>31485245.74</v>
       </c>
       <c r="F216" s="12" t="n">
-        <v>6123706.92</v>
+        <v>17446676.21</v>
       </c>
       <c r="G216" s="12" t="n">
-        <v>29987724.42</v>
+        <v>14038569.74</v>
       </c>
     </row>
     <row r="217" spans="1:7" ht="16.5" customHeight="1">
       <c r="A217" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B217" s="7">
-        <v>46099</v>
-      </c>
-      <c r="C217" s="9">
-        <v/>
+        <v>46113</v>
+      </c>
+      <c r="C217" s="9" t="n">
+        <v>35.00</v>
       </c>
       <c r="D217" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E217" s="12" t="n">
-        <v>36111431.42</v>
+        <v>31485245.74</v>
       </c>
       <c r="F217" s="12" t="n">
-        <v>6123706.92</v>
+        <v>17446676.21</v>
       </c>
       <c r="G217" s="12" t="n">
-        <v>29987724.42</v>
+        <v>14038569.74</v>
       </c>
     </row>
     <row r="218" spans="1:7" ht="16.5" customHeight="1">
       <c r="A218" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B218" s="7">
-        <v>46085</v>
+        <v>46100</v>
       </c>
       <c r="C218" s="9" t="n">
-        <v>90.00</v>
+        <v>75.00</v>
       </c>
       <c r="D218" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E218" s="12" t="n">
-        <v>1004599.27</v>
+        <v>36111431.42</v>
       </c>
       <c r="F218" s="12" t="n">
-        <v>840417.82</v>
+        <v>6123706.92</v>
       </c>
       <c r="G218" s="12" t="n">
-        <v>164181.45</v>
+        <v>29987724.42</v>
       </c>
     </row>
     <row r="219" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A219" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B219" s="6">
-        <v>46101</v>
-      </c>
-      <c r="C219" s="8" t="n">
-        <v>90.00</v>
-      </c>
-      <c r="D219" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="E219" s="11" t="n">
-        <v>1626262.86</v>
-      </c>
-      <c r="F219" s="11" t="n">
-        <v>1680835.64</v>
-      </c>
-      <c r="G219" s="11" t="n">
-        <v>-54572.78</v>
+      <c r="A219" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B219" s="7">
+        <v>46099</v>
+      </c>
+      <c r="C219" s="9">
+        <v/>
+      </c>
+      <c r="D219" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="E219" s="12" t="n">
+        <v>36111431.42</v>
+      </c>
+      <c r="F219" s="12" t="n">
+        <v>6123706.92</v>
+      </c>
+      <c r="G219" s="12" t="n">
+        <v>29987724.42</v>
       </c>
     </row>
     <row r="220" spans="1:7" ht="16.5" customHeight="1">
       <c r="A220" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B220" s="7">
-        <v>46091</v>
+        <v>46085</v>
       </c>
       <c r="C220" s="9" t="n">
         <v>90.00</v>
       </c>
       <c r="D220" s="3" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E220" s="12" t="n">
-        <v>777981.56</v>
+        <v>1004599.27</v>
       </c>
       <c r="F220" s="12" t="n">
-        <v>526208.91</v>
+        <v>840417.82</v>
       </c>
       <c r="G220" s="12" t="n">
-        <v>251772.65</v>
+        <v>164181.45</v>
       </c>
     </row>
     <row r="221" spans="1:7" ht="16.5" customHeight="1">
       <c r="A221" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B221" s="6">
-        <v>46132</v>
+        <v>46101</v>
       </c>
       <c r="C221" s="8" t="n">
-        <v>5.00</v>
+        <v>90.00</v>
       </c>
       <c r="D221" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E221" s="11" t="n">
-        <v>82174.71</v>
+        <v>1626262.86</v>
       </c>
       <c r="F221" s="11" t="n">
-        <v>252125.35</v>
+        <v>1680835.64</v>
       </c>
       <c r="G221" s="11" t="n">
-        <v>-169950.29</v>
+        <v>-54572.78</v>
       </c>
     </row>
     <row r="222" spans="1:7" ht="16.5" customHeight="1">
       <c r="A222" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B222" s="7">
-        <v>46154</v>
+        <v>46091</v>
       </c>
       <c r="C222" s="9" t="n">
-        <v>28.00</v>
+        <v>90.00</v>
       </c>
       <c r="D222" s="3" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E222" s="12" t="n">
-        <v>17728563.67</v>
+        <v>777981.56</v>
       </c>
       <c r="F222" s="12" t="n">
-        <v>5964706.92</v>
+        <v>526208.91</v>
       </c>
       <c r="G222" s="12" t="n">
-        <v>11763856.75</v>
+        <v>251772.65</v>
       </c>
     </row>
     <row r="223" spans="1:7" ht="16.5" customHeight="1">
-      <c r="A223" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="B223" s="7">
-        <v>46153</v>
-      </c>
-      <c r="C223" s="9" t="n">
-        <v>24.00</v>
-      </c>
-      <c r="D223" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="E223" s="12" t="n">
-        <v>17728563.67</v>
-      </c>
-      <c r="F223" s="12" t="n">
-        <v>5964706.92</v>
-      </c>
-      <c r="G223" s="12" t="n">
-        <v>11763856.75</v>
+      <c r="A223" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B223" s="6">
+        <v>46132</v>
+      </c>
+      <c r="C223" s="8" t="n">
+        <v>5.00</v>
+      </c>
+      <c r="D223" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E223" s="11" t="n">
+        <v>82174.71</v>
+      </c>
+      <c r="F223" s="11" t="n">
+        <v>252125.35</v>
+      </c>
+      <c r="G223" s="11" t="n">
+        <v>-169950.29</v>
       </c>
     </row>
     <row r="224" spans="1:7" ht="16.5" customHeight="1">
       <c r="A224" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B224" s="7">
         <v>46154</v>
       </c>
       <c r="C224" s="9" t="n">
-        <v>72.22</v>
+        <v>28.00</v>
       </c>
       <c r="D224" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E224" s="12" t="n">
-        <v>1465200389.67</v>
+        <v>17728563.67</v>
       </c>
       <c r="F224" s="12" t="n">
-        <v>91732232.52</v>
+        <v>5964706.92</v>
       </c>
       <c r="G224" s="12" t="n">
-        <v>1373468157.15</v>
+        <v>11763856.75</v>
       </c>
     </row>
     <row r="225" spans="1:7" ht="16.5" customHeight="1">
       <c r="A225" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B225" s="7">
-        <v>46149</v>
+        <v>46153</v>
       </c>
       <c r="C225" s="9" t="n">
-        <v>72.04</v>
+        <v>24.00</v>
       </c>
       <c r="D225" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E225" s="12" t="n">
-        <v>1465200389.67</v>
+        <v>17728563.67</v>
       </c>
       <c r="F225" s="12" t="n">
-        <v>91732232.52</v>
+        <v>5964706.92</v>
       </c>
       <c r="G225" s="12" t="n">
-        <v>1373468157.15</v>
+        <v>11763856.75</v>
       </c>
     </row>
     <row r="226" spans="1:7" ht="16.5" customHeight="1">
@@ -6466,10 +6466,10 @@
         <v>123</v>
       </c>
       <c r="B226" s="7">
-        <v>46148</v>
+        <v>46154</v>
       </c>
       <c r="C226" s="9" t="n">
-        <v>71.66</v>
+        <v>72.22</v>
       </c>
       <c r="D226" s="3" t="s">
         <v>253</v>
@@ -6489,10 +6489,10 @@
         <v>123</v>
       </c>
       <c r="B227" s="7">
-        <v>46142</v>
+        <v>46149</v>
       </c>
       <c r="C227" s="9" t="n">
-        <v>71.22</v>
+        <v>72.04</v>
       </c>
       <c r="D227" s="3" t="s">
         <v>253</v>
@@ -6512,10 +6512,10 @@
         <v>123</v>
       </c>
       <c r="B228" s="7">
-        <v>46141</v>
+        <v>46148</v>
       </c>
       <c r="C228" s="9" t="n">
-        <v>71.12</v>
+        <v>71.66</v>
       </c>
       <c r="D228" s="3" t="s">
         <v>253</v>
@@ -6535,10 +6535,10 @@
         <v>123</v>
       </c>
       <c r="B229" s="7">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c r="C229" s="9" t="n">
-        <v>71.42</v>
+        <v>71.22</v>
       </c>
       <c r="D229" s="3" t="s">
         <v>253</v>
@@ -6558,10 +6558,10 @@
         <v>123</v>
       </c>
       <c r="B230" s="7">
-        <v>46134</v>
+        <v>46141</v>
       </c>
       <c r="C230" s="9" t="n">
-        <v>71.19</v>
+        <v>71.12</v>
       </c>
       <c r="D230" s="3" t="s">
         <v>253</v>
@@ -6581,10 +6581,10 @@
         <v>123</v>
       </c>
       <c r="B231" s="7">
-        <v>46133</v>
+        <v>46139</v>
       </c>
       <c r="C231" s="9" t="n">
-        <v>71.01</v>
+        <v>71.42</v>
       </c>
       <c r="D231" s="3" t="s">
         <v>253</v>
@@ -6604,10 +6604,10 @@
         <v>123</v>
       </c>
       <c r="B232" s="7">
-        <v>46126</v>
+        <v>46134</v>
       </c>
       <c r="C232" s="9" t="n">
-        <v>70.71</v>
+        <v>71.19</v>
       </c>
       <c r="D232" s="3" t="s">
         <v>253</v>
@@ -6627,10 +6627,10 @@
         <v>123</v>
       </c>
       <c r="B233" s="7">
-        <v>46120</v>
+        <v>46133</v>
       </c>
       <c r="C233" s="9" t="n">
-        <v>70.58</v>
+        <v>71.01</v>
       </c>
       <c r="D233" s="3" t="s">
         <v>253</v>
@@ -6650,10 +6650,10 @@
         <v>123</v>
       </c>
       <c r="B234" s="7">
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="C234" s="9" t="n">
-        <v>68.58</v>
+        <v>70.71</v>
       </c>
       <c r="D234" s="3" t="s">
         <v>253</v>
@@ -6673,10 +6673,10 @@
         <v>123</v>
       </c>
       <c r="B235" s="7">
-        <v>46107</v>
+        <v>46120</v>
       </c>
       <c r="C235" s="9" t="n">
-        <v>67.28</v>
+        <v>70.58</v>
       </c>
       <c r="D235" s="3" t="s">
         <v>253</v>
@@ -6696,10 +6696,10 @@
         <v>123</v>
       </c>
       <c r="B236" s="7">
-        <v>46099</v>
+        <v>46115</v>
       </c>
       <c r="C236" s="9" t="n">
-        <v>66.60</v>
+        <v>68.58</v>
       </c>
       <c r="D236" s="3" t="s">
         <v>253</v>
@@ -6719,10 +6719,10 @@
         <v>123</v>
       </c>
       <c r="B237" s="7">
-        <v>46098</v>
+        <v>46107</v>
       </c>
       <c r="C237" s="9" t="n">
-        <v>66.60</v>
+        <v>67.28</v>
       </c>
       <c r="D237" s="3" t="s">
         <v>253</v>
@@ -6742,10 +6742,10 @@
         <v>123</v>
       </c>
       <c r="B238" s="7">
-        <v>46097</v>
+        <v>46099</v>
       </c>
       <c r="C238" s="9" t="n">
-        <v>65.90</v>
+        <v>66.60</v>
       </c>
       <c r="D238" s="3" t="s">
         <v>253</v>
@@ -6765,10 +6765,10 @@
         <v>123</v>
       </c>
       <c r="B239" s="7">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="C239" s="9" t="n">
-        <v>65.10</v>
+        <v>66.60</v>
       </c>
       <c r="D239" s="3" t="s">
         <v>253</v>
@@ -6788,10 +6788,10 @@
         <v>123</v>
       </c>
       <c r="B240" s="7">
-        <v>46093</v>
+        <v>46097</v>
       </c>
       <c r="C240" s="9" t="n">
-        <v>64.20</v>
+        <v>65.90</v>
       </c>
       <c r="D240" s="3" t="s">
         <v>253</v>
@@ -6811,10 +6811,10 @@
         <v>123</v>
       </c>
       <c r="B241" s="7">
-        <v>46092</v>
+        <v>46094</v>
       </c>
       <c r="C241" s="9" t="n">
-        <v>63.20</v>
+        <v>65.10</v>
       </c>
       <c r="D241" s="3" t="s">
         <v>253</v>
@@ -6834,10 +6834,10 @@
         <v>123</v>
       </c>
       <c r="B242" s="7">
-        <v>46091</v>
+        <v>46093</v>
       </c>
       <c r="C242" s="9" t="n">
-        <v>61.70</v>
+        <v>64.20</v>
       </c>
       <c r="D242" s="3" t="s">
         <v>253</v>
@@ -6857,10 +6857,10 @@
         <v>123</v>
       </c>
       <c r="B243" s="7">
-        <v>46052</v>
+        <v>46092</v>
       </c>
       <c r="C243" s="9" t="n">
-        <v>59.64</v>
+        <v>63.20</v>
       </c>
       <c r="D243" s="3" t="s">
         <v>253</v>
@@ -6880,10 +6880,10 @@
         <v>123</v>
       </c>
       <c r="B244" s="7">
-        <v>46022</v>
+        <v>46091</v>
       </c>
       <c r="C244" s="9" t="n">
-        <v>59.64</v>
+        <v>61.70</v>
       </c>
       <c r="D244" s="3" t="s">
         <v>253</v>
@@ -6900,48 +6900,48 @@
     </row>
     <row r="245" spans="1:7" ht="16.5" customHeight="1">
       <c r="A245" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B245" s="7">
-        <v>46184</v>
+        <v>46052</v>
       </c>
       <c r="C245" s="9" t="n">
-        <v>66.46</v>
+        <v>59.64</v>
       </c>
       <c r="D245" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E245" s="12" t="n">
-        <v>826455966.23</v>
+        <v>1465200389.67</v>
       </c>
       <c r="F245" s="12" t="n">
-        <v>89086834.51</v>
+        <v>91732232.52</v>
       </c>
       <c r="G245" s="12" t="n">
-        <v>737369131.72</v>
+        <v>1373468157.15</v>
       </c>
     </row>
     <row r="246" spans="1:7" ht="16.5" customHeight="1">
       <c r="A246" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B246" s="7">
-        <v>46183</v>
+        <v>46022</v>
       </c>
       <c r="C246" s="9" t="n">
-        <v>66.10</v>
+        <v>59.64</v>
       </c>
       <c r="D246" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E246" s="12" t="n">
-        <v>826455966.23</v>
+        <v>1465200389.67</v>
       </c>
       <c r="F246" s="12" t="n">
-        <v>89086834.51</v>
+        <v>91732232.52</v>
       </c>
       <c r="G246" s="12" t="n">
-        <v>737369131.72</v>
+        <v>1373468157.15</v>
       </c>
     </row>
     <row r="247" spans="1:7" ht="16.5" customHeight="1">
@@ -6949,10 +6949,10 @@
         <v>124</v>
       </c>
       <c r="B247" s="7">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="C247" s="9" t="n">
-        <v>65.56</v>
+        <v>66.46</v>
       </c>
       <c r="D247" s="3" t="s">
         <v>254</v>
@@ -6972,10 +6972,10 @@
         <v>124</v>
       </c>
       <c r="B248" s="7">
-        <v>46181</v>
+        <v>46183</v>
       </c>
       <c r="C248" s="9" t="n">
-        <v>65.30</v>
+        <v>66.10</v>
       </c>
       <c r="D248" s="3" t="s">
         <v>254</v>
@@ -6995,10 +6995,10 @@
         <v>124</v>
       </c>
       <c r="B249" s="7">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="C249" s="9" t="n">
-        <v>64.89</v>
+        <v>65.56</v>
       </c>
       <c r="D249" s="3" t="s">
         <v>254</v>
@@ -7018,10 +7018,10 @@
         <v>124</v>
       </c>
       <c r="B250" s="7">
-        <v>46175</v>
+        <v>46181</v>
       </c>
       <c r="C250" s="9" t="n">
-        <v>64.78</v>
+        <v>65.30</v>
       </c>
       <c r="D250" s="3" t="s">
         <v>254</v>
@@ -7041,10 +7041,10 @@
         <v>124</v>
       </c>
       <c r="B251" s="7">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="C251" s="9" t="n">
-        <v>64.10</v>
+        <v>64.89</v>
       </c>
       <c r="D251" s="3" t="s">
         <v>254</v>
@@ -7064,10 +7064,10 @@
         <v>124</v>
       </c>
       <c r="B252" s="7">
-        <v>46170</v>
+        <v>46175</v>
       </c>
       <c r="C252" s="9" t="n">
-        <v>63.46</v>
+        <v>64.78</v>
       </c>
       <c r="D252" s="3" t="s">
         <v>254</v>
@@ -7087,10 +7087,10 @@
         <v>124</v>
       </c>
       <c r="B253" s="7">
-        <v>46169</v>
+        <v>46174</v>
       </c>
       <c r="C253" s="9" t="n">
-        <v>63.00</v>
+        <v>64.10</v>
       </c>
       <c r="D253" s="3" t="s">
         <v>254</v>
@@ -7110,10 +7110,10 @@
         <v>124</v>
       </c>
       <c r="B254" s="7">
-        <v>46163</v>
+        <v>46170</v>
       </c>
       <c r="C254" s="9" t="n">
-        <v>63.00</v>
+        <v>63.46</v>
       </c>
       <c r="D254" s="3" t="s">
         <v>254</v>
@@ -7133,7 +7133,7 @@
         <v>124</v>
       </c>
       <c r="B255" s="7">
-        <v>46161</v>
+        <v>46169</v>
       </c>
       <c r="C255" s="9" t="n">
         <v>63.00</v>
@@ -7156,7 +7156,7 @@
         <v>124</v>
       </c>
       <c r="B256" s="7">
-        <v>46160</v>
+        <v>46163</v>
       </c>
       <c r="C256" s="9" t="n">
         <v>63.00</v>
@@ -7179,10 +7179,10 @@
         <v>124</v>
       </c>
       <c r="B257" s="7">
-        <v>46156</v>
+        <v>46161</v>
       </c>
       <c r="C257" s="9" t="n">
-        <v>62.00</v>
+        <v>63.00</v>
       </c>
       <c r="D257" s="3" t="s">
         <v>254</v>
@@ -7202,10 +7202,10 @@
         <v>124</v>
       </c>
       <c r="B258" s="7">
-        <v>46155</v>
+        <v>46160</v>
       </c>
       <c r="C258" s="9" t="n">
-        <v>62.00</v>
+        <v>63.00</v>
       </c>
       <c r="D258" s="3" t="s">
         <v>254</v>
@@ -7225,7 +7225,7 @@
         <v>124</v>
       </c>
       <c r="B259" s="7">
-        <v>46149</v>
+        <v>46156</v>
       </c>
       <c r="C259" s="9" t="n">
         <v>62.00</v>
@@ -7248,10 +7248,10 @@
         <v>124</v>
       </c>
       <c r="B260" s="7">
-        <v>46120</v>
+        <v>46155</v>
       </c>
       <c r="C260" s="9" t="n">
-        <v>61.56</v>
+        <v>62.00</v>
       </c>
       <c r="D260" s="3" t="s">
         <v>254</v>
@@ -7271,10 +7271,10 @@
         <v>124</v>
       </c>
       <c r="B261" s="7">
-        <v>46119</v>
+        <v>46149</v>
       </c>
       <c r="C261" s="9" t="n">
-        <v>61.00</v>
+        <v>62.00</v>
       </c>
       <c r="D261" s="3" t="s">
         <v>254</v>
@@ -7294,10 +7294,10 @@
         <v>124</v>
       </c>
       <c r="B262" s="7">
-        <v>46114</v>
+        <v>46120</v>
       </c>
       <c r="C262" s="9" t="n">
-        <v>60.00</v>
+        <v>61.56</v>
       </c>
       <c r="D262" s="3" t="s">
         <v>254</v>
@@ -7317,10 +7317,10 @@
         <v>124</v>
       </c>
       <c r="B263" s="7">
-        <v>46112</v>
+        <v>46119</v>
       </c>
       <c r="C263" s="9" t="n">
-        <v>56.83</v>
+        <v>61.00</v>
       </c>
       <c r="D263" s="3" t="s">
         <v>254</v>
@@ -7340,10 +7340,10 @@
         <v>124</v>
       </c>
       <c r="B264" s="7">
-        <v>46111</v>
+        <v>46114</v>
       </c>
       <c r="C264" s="9" t="n">
-        <v>56.00</v>
+        <v>60.00</v>
       </c>
       <c r="D264" s="3" t="s">
         <v>254</v>
@@ -7363,10 +7363,10 @@
         <v>124</v>
       </c>
       <c r="B265" s="7">
-        <v>46108</v>
+        <v>46112</v>
       </c>
       <c r="C265" s="9" t="n">
-        <v>56.00</v>
+        <v>56.83</v>
       </c>
       <c r="D265" s="3" t="s">
         <v>254</v>
@@ -7386,10 +7386,10 @@
         <v>124</v>
       </c>
       <c r="B266" s="7">
-        <v>46105</v>
+        <v>46111</v>
       </c>
       <c r="C266" s="9" t="n">
-        <v>56.00</v>
+        <v>56.43</v>
       </c>
       <c r="D266" s="3" t="s">
         <v>254</v>
@@ -7409,10 +7409,10 @@
         <v>124</v>
       </c>
       <c r="B267" s="7">
-        <v>46090</v>
+        <v>46108</v>
       </c>
       <c r="C267" s="9" t="n">
-        <v>56.00</v>
+        <v>55.81</v>
       </c>
       <c r="D267" s="3" t="s">
         <v>254</v>
@@ -7432,10 +7432,10 @@
         <v>124</v>
       </c>
       <c r="B268" s="7">
-        <v>46085</v>
+        <v>46105</v>
       </c>
       <c r="C268" s="9" t="n">
-        <v>55.00</v>
+        <v>55.70</v>
       </c>
       <c r="D268" s="3" t="s">
         <v>254</v>
@@ -7455,10 +7455,10 @@
         <v>124</v>
       </c>
       <c r="B269" s="7">
-        <v>46084</v>
+        <v>46090</v>
       </c>
       <c r="C269" s="9" t="n">
-        <v>54.00</v>
+        <v>55.58</v>
       </c>
       <c r="D269" s="3" t="s">
         <v>254</v>
@@ -7478,10 +7478,10 @@
         <v>124</v>
       </c>
       <c r="B270" s="7">
-        <v>46080</v>
+        <v>46085</v>
       </c>
       <c r="C270" s="9" t="n">
-        <v>53.21</v>
+        <v>55.08</v>
       </c>
       <c r="D270" s="3" t="s">
         <v>254</v>
@@ -7501,10 +7501,10 @@
         <v>124</v>
       </c>
       <c r="B271" s="7">
-        <v>46079</v>
+        <v>46084</v>
       </c>
       <c r="C271" s="9" t="n">
-        <v>49.00</v>
+        <v>54.41</v>
       </c>
       <c r="D271" s="3" t="s">
         <v>254</v>
@@ -7524,10 +7524,10 @@
         <v>124</v>
       </c>
       <c r="B272" s="7">
-        <v>46052</v>
+        <v>46080</v>
       </c>
       <c r="C272" s="9" t="n">
-        <v>44.21</v>
+        <v>53.21</v>
       </c>
       <c r="D272" s="3" t="s">
         <v>254</v>
@@ -7547,10 +7547,10 @@
         <v>124</v>
       </c>
       <c r="B273" s="7">
-        <v>46022</v>
+        <v>46079</v>
       </c>
       <c r="C273" s="9" t="n">
-        <v>44.21</v>
+        <v>48.72</v>
       </c>
       <c r="D273" s="3" t="s">
         <v>254</v>
@@ -7567,48 +7567,48 @@
     </row>
     <row r="274" spans="1:7" ht="16.5" customHeight="1">
       <c r="A274" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B274" s="7">
-        <v>46115</v>
+        <v>46052</v>
       </c>
       <c r="C274" s="9" t="n">
-        <v>92.06</v>
+        <v>44.21</v>
       </c>
       <c r="D274" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E274" s="12" t="n">
-        <v>214681273.28</v>
+        <v>826455966.23</v>
       </c>
       <c r="F274" s="12" t="n">
-        <v>72980322.66</v>
+        <v>89086834.51</v>
       </c>
       <c r="G274" s="12" t="n">
-        <v>141700950.62</v>
+        <v>737369131.72</v>
       </c>
     </row>
     <row r="275" spans="1:7" ht="16.5" customHeight="1">
       <c r="A275" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B275" s="7">
-        <v>46106</v>
+        <v>46022</v>
       </c>
       <c r="C275" s="9" t="n">
-        <v>89.66</v>
+        <v>43.00</v>
       </c>
       <c r="D275" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E275" s="12" t="n">
-        <v>214681273.28</v>
+        <v>826455966.23</v>
       </c>
       <c r="F275" s="12" t="n">
-        <v>72980322.66</v>
+        <v>89086834.51</v>
       </c>
       <c r="G275" s="12" t="n">
-        <v>141700950.62</v>
+        <v>737369131.72</v>
       </c>
     </row>
     <row r="276" spans="1:7" ht="16.5" customHeight="1">
@@ -7616,10 +7616,10 @@
         <v>125</v>
       </c>
       <c r="B276" s="7">
-        <v>46080</v>
+        <v>46115</v>
       </c>
       <c r="C276" s="9" t="n">
-        <v>87.46</v>
+        <v>92.06</v>
       </c>
       <c r="D276" s="3" t="s">
         <v>255</v>
@@ -7639,10 +7639,10 @@
         <v>125</v>
       </c>
       <c r="B277" s="7">
-        <v>46049</v>
+        <v>46106</v>
       </c>
       <c r="C277" s="9" t="n">
-        <v>87.46</v>
+        <v>89.66</v>
       </c>
       <c r="D277" s="3" t="s">
         <v>255</v>
@@ -7662,10 +7662,10 @@
         <v>125</v>
       </c>
       <c r="B278" s="7">
-        <v>46043</v>
+        <v>46080</v>
       </c>
       <c r="C278" s="9" t="n">
-        <v>86.48</v>
+        <v>87.46</v>
       </c>
       <c r="D278" s="3" t="s">
         <v>255</v>
@@ -7685,10 +7685,10 @@
         <v>125</v>
       </c>
       <c r="B279" s="7">
-        <v>46035</v>
+        <v>46049</v>
       </c>
       <c r="C279" s="9" t="n">
-        <v>85.65</v>
+        <v>87.46</v>
       </c>
       <c r="D279" s="3" t="s">
         <v>255</v>
@@ -7708,10 +7708,10 @@
         <v>125</v>
       </c>
       <c r="B280" s="7">
-        <v>46034</v>
+        <v>46043</v>
       </c>
       <c r="C280" s="9" t="n">
-        <v>85.00</v>
+        <v>86.48</v>
       </c>
       <c r="D280" s="3" t="s">
         <v>255</v>
@@ -7731,10 +7731,10 @@
         <v>125</v>
       </c>
       <c r="B281" s="7">
-        <v>46015</v>
+        <v>46035</v>
       </c>
       <c r="C281" s="9" t="n">
-        <v>84.43</v>
+        <v>85.65</v>
       </c>
       <c r="D281" s="3" t="s">
         <v>255</v>
@@ -7751,48 +7751,48 @@
     </row>
     <row r="282" spans="1:7" ht="16.5" customHeight="1">
       <c r="A282" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B282" s="7">
-        <v>46105</v>
+        <v>46034</v>
       </c>
       <c r="C282" s="9" t="n">
-        <v>81.62</v>
+        <v>85.00</v>
       </c>
       <c r="D282" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E282" s="12" t="n">
-        <v>475052441.17</v>
+        <v>214681273.28</v>
       </c>
       <c r="F282" s="12" t="n">
-        <v>18549774.22</v>
+        <v>72980322.66</v>
       </c>
       <c r="G282" s="12" t="n">
-        <v>456502666.95</v>
+        <v>141700950.62</v>
       </c>
     </row>
     <row r="283" spans="1:7" ht="16.5" customHeight="1">
       <c r="A283" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B283" s="7">
-        <v>46104</v>
+        <v>46015</v>
       </c>
       <c r="C283" s="9" t="n">
-        <v>81.12</v>
+        <v>84.43</v>
       </c>
       <c r="D283" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E283" s="12" t="n">
-        <v>475052441.17</v>
+        <v>214681273.28</v>
       </c>
       <c r="F283" s="12" t="n">
-        <v>18549774.22</v>
+        <v>72980322.66</v>
       </c>
       <c r="G283" s="12" t="n">
-        <v>456502666.95</v>
+        <v>141700950.62</v>
       </c>
     </row>
     <row r="284" spans="1:7" ht="16.5" customHeight="1">
@@ -7800,10 +7800,10 @@
         <v>126</v>
       </c>
       <c r="B284" s="7">
-        <v>46097</v>
+        <v>46105</v>
       </c>
       <c r="C284" s="9" t="n">
-        <v>80.12</v>
+        <v>81.62</v>
       </c>
       <c r="D284" s="3" t="s">
         <v>256</v>
@@ -7823,10 +7823,10 @@
         <v>126</v>
       </c>
       <c r="B285" s="7">
-        <v>46087</v>
+        <v>46104</v>
       </c>
       <c r="C285" s="9" t="n">
-        <v>79.22</v>
+        <v>81.12</v>
       </c>
       <c r="D285" s="3" t="s">
         <v>256</v>
@@ -7846,10 +7846,10 @@
         <v>126</v>
       </c>
       <c r="B286" s="7">
-        <v>46043</v>
+        <v>46097</v>
       </c>
       <c r="C286" s="9" t="n">
-        <v>78.52</v>
+        <v>80.12</v>
       </c>
       <c r="D286" s="3" t="s">
         <v>256</v>
@@ -7869,10 +7869,10 @@
         <v>126</v>
       </c>
       <c r="B287" s="7">
-        <v>46037</v>
+        <v>46087</v>
       </c>
       <c r="C287" s="9" t="n">
-        <v>77.52</v>
+        <v>79.22</v>
       </c>
       <c r="D287" s="3" t="s">
         <v>256</v>
@@ -7892,10 +7892,10 @@
         <v>126</v>
       </c>
       <c r="B288" s="7">
-        <v>46030</v>
+        <v>46043</v>
       </c>
       <c r="C288" s="9" t="n">
-        <v>77.32</v>
+        <v>78.52</v>
       </c>
       <c r="D288" s="3" t="s">
         <v>256</v>
@@ -7915,10 +7915,10 @@
         <v>126</v>
       </c>
       <c r="B289" s="7">
-        <v>46029</v>
+        <v>46037</v>
       </c>
       <c r="C289" s="9" t="n">
-        <v>76.77</v>
+        <v>77.52</v>
       </c>
       <c r="D289" s="3" t="s">
         <v>256</v>
@@ -7938,10 +7938,10 @@
         <v>126</v>
       </c>
       <c r="B290" s="7">
-        <v>46021</v>
+        <v>46030</v>
       </c>
       <c r="C290" s="9" t="n">
-        <v>76.46</v>
+        <v>77.32</v>
       </c>
       <c r="D290" s="3" t="s">
         <v>256</v>
@@ -7958,48 +7958,48 @@
     </row>
     <row r="291" spans="1:7" ht="16.5" customHeight="1">
       <c r="A291" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B291" s="7">
-        <v>46042</v>
+        <v>46029</v>
       </c>
       <c r="C291" s="9" t="n">
-        <v>7.00</v>
+        <v>76.77</v>
       </c>
       <c r="D291" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E291" s="12" t="n">
-        <v>38850000.00</v>
+        <v>475052441.17</v>
       </c>
       <c r="F291" s="12" t="n">
-        <v>21642692.04</v>
+        <v>18549774.22</v>
       </c>
       <c r="G291" s="12" t="n">
-        <v>17207307.96</v>
+        <v>456502666.95</v>
       </c>
     </row>
     <row r="292" spans="1:7" ht="16.5" customHeight="1">
       <c r="A292" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B292" s="7">
-        <v>46041</v>
+        <v>46021</v>
       </c>
       <c r="C292" s="9" t="n">
-        <v>5.00</v>
+        <v>76.46</v>
       </c>
       <c r="D292" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E292" s="12" t="n">
-        <v>38850000.00</v>
+        <v>475052441.17</v>
       </c>
       <c r="F292" s="12" t="n">
-        <v>21642692.04</v>
+        <v>18549774.22</v>
       </c>
       <c r="G292" s="12" t="n">
-        <v>17207307.96</v>
+        <v>456502666.95</v>
       </c>
     </row>
     <row r="293" spans="1:7" ht="16.5" customHeight="1">
@@ -8007,10 +8007,10 @@
         <v>127</v>
       </c>
       <c r="B293" s="7">
-        <v>46038</v>
+        <v>46042</v>
       </c>
       <c r="C293" s="9" t="n">
-        <v>5.00</v>
+        <v>7.00</v>
       </c>
       <c r="D293" s="3" t="s">
         <v>257</v>
@@ -8030,7 +8030,7 @@
         <v>127</v>
       </c>
       <c r="B294" s="7">
-        <v>46037</v>
+        <v>46041</v>
       </c>
       <c r="C294" s="9" t="n">
         <v>5.00</v>
@@ -8053,10 +8053,10 @@
         <v>127</v>
       </c>
       <c r="B295" s="7">
-        <v>46036</v>
+        <v>46038</v>
       </c>
       <c r="C295" s="9" t="n">
-        <v>2.00</v>
+        <v>5.00</v>
       </c>
       <c r="D295" s="3" t="s">
         <v>257</v>
@@ -8076,10 +8076,10 @@
         <v>127</v>
       </c>
       <c r="B296" s="7">
-        <v>46030</v>
+        <v>46037</v>
       </c>
       <c r="C296" s="9" t="n">
-        <v>1.00</v>
+        <v>5.00</v>
       </c>
       <c r="D296" s="3" t="s">
         <v>257</v>
@@ -8094,34 +8094,80 @@
         <v>17207307.96</v>
       </c>
     </row>
-    <row r="297" spans="1:7" ht="1.5" customHeight="1">
-      <c r="A297" s="4"/>
-      <c r="B297" s="4"/>
-      <c r="C297" s="4"/>
-      <c r="D297" s="4"/>
-      <c r="E297" s="13"/>
-      <c r="F297" s="13"/>
-      <c r="G297" s="16"/>
-    </row>
-    <row r="298" spans="1:7" ht="14.25" customHeight="1">
-      <c r="A298" s="5"/>
-      <c r="B298" s="5"/>
-      <c r="C298" s="5"/>
-      <c r="D298" s="5"/>
-      <c r="E298" s="14" t="n">
-        <v>67725720076.33</v>
-      </c>
-      <c r="F298" s="15" t="n">
-        <v>8288437054.88</v>
-      </c>
-      <c r="G298" s="15" t="n">
-        <v>59284933549.81</v>
+    <row r="297" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A297" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B297" s="7">
+        <v>46036</v>
+      </c>
+      <c r="C297" s="9" t="n">
+        <v>2.00</v>
+      </c>
+      <c r="D297" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="E297" s="12" t="n">
+        <v>38850000.00</v>
+      </c>
+      <c r="F297" s="12" t="n">
+        <v>21642692.04</v>
+      </c>
+      <c r="G297" s="12" t="n">
+        <v>17207307.96</v>
+      </c>
+    </row>
+    <row r="298" spans="1:7" ht="16.5" customHeight="1">
+      <c r="A298" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B298" s="7">
+        <v>46030</v>
+      </c>
+      <c r="C298" s="9" t="n">
+        <v>1.00</v>
+      </c>
+      <c r="D298" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="E298" s="12" t="n">
+        <v>38850000.00</v>
+      </c>
+      <c r="F298" s="12" t="n">
+        <v>21642692.04</v>
+      </c>
+      <c r="G298" s="12" t="n">
+        <v>17207307.96</v>
+      </c>
+    </row>
+    <row r="299" spans="1:7" ht="1.5" customHeight="1">
+      <c r="A299" s="4"/>
+      <c r="B299" s="4"/>
+      <c r="C299" s="4"/>
+      <c r="D299" s="4"/>
+      <c r="E299" s="13"/>
+      <c r="F299" s="13"/>
+      <c r="G299" s="16"/>
+    </row>
+    <row r="300" spans="1:7" ht="14.25" customHeight="1">
+      <c r="A300" s="5"/>
+      <c r="B300" s="5"/>
+      <c r="C300" s="5"/>
+      <c r="D300" s="5"/>
+      <c r="E300" s="14" t="n">
+        <v>67758669637.21</v>
+      </c>
+      <c r="F300" s="15" t="n">
+        <v>8320650851.85</v>
+      </c>
+      <c r="G300" s="15" t="n">
+        <v>59285669313.72</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A297:D297"/>
-    <mergeCell ref="A298:D298"/>
+    <mergeCell ref="A299:D299"/>
+    <mergeCell ref="A300:D300"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>